<commit_message>
Aprova 100 fotos flagueadas so por nome de rua divergente
Casos conferidos manualmente pelo usuario (cod_id 221621781,
219991739 e outros do mesmo padrao): o motivo do flag era so
nome de rua muito diferente entre o endereco reportado pelo
Street View e o cod_id escolhido -- tipico de esquina, onde o
endereco mais proximo legitimamente varia sem ser erro de match.
Nao mexe nos casos flagueados por discordancia de distancia/rumo,
esses continuam em BAIXA CONFIANCA - REVISAO ate confirmacao.

POSTES UTILIZADOS/: 81 movidos pra POSTE UTILIZADO - OK, 19 pra
ESQUINA - OK (sem o !! no nome, ja aprovados).

RELATORIOS/links_postes_processados.xlsx: pasta_atual atualizada
pros 100 cod_id movidos; removida 1 linha duplicada do cod_id
219991739 (dois links antigos resolviam pro mesmo poste, so um
tinha arquivo fisico -- mantida a linha correta).

RELATORIOS/confirmar_manual.xlsx e duplicados_para_validar.xlsx:
relatorios do lote de 511 links processado antes, ainda nao
commitados.
</commit_message>
<xml_diff>
--- a/RELATORIOS/confirmar_manual.xlsx
+++ b/RELATORIOS/confirmar_manual.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G249"/>
+  <dimension ref="A1:G389"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -7904,6 +7904,4206 @@
         </is>
       </c>
       <c r="G249" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>219386697</t>
+        </is>
+      </c>
+      <c r="B250" t="n">
+        <v>928</v>
+      </c>
+      <c r="C250" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.6075741,-46.9455072,3a,90y,106.93h,121.72t/data=!3m7!1e1!3m5!1sXBYexVciCLGrEILQKLLmyw!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-31.717366152706177%26panoid%3DXBYexVciCLGrEILQKLLmyw%26yaw%3D106.92727030292335!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>AVENIDA JOAO PAULO II 2515, 2515, FERTIZA</t>
+        </is>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>confirmar - poste mais proximo (5.4m) tem 68 graus de diferenca de rumo, mas esta perto o suficiente pra ser so ruido de GPS</t>
+        </is>
+      </c>
+      <c r="G250" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>220247556</t>
+        </is>
+      </c>
+      <c r="B251" t="n">
+        <v>929</v>
+      </c>
+      <c r="C251" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.6073938,-46.9454412,3a,90y,47.06h,112.79t/data=!3m7!1e1!3m5!1sHwX9-m6b6MMiu6IIevnpmQ!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-22.79461445357704%26panoid%3DHwX9-m6b6MMiu6IIevnpmQ%26yaw%3D47.058643482662525!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>RUA ARGENTINA DE OLIVEIRA FERREIRA 185, 185, FERTIZA</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>ATENCAO nome de rua muito diferente: Street View diz o endereco e '3362 Av. João Paulo II', cod_id escolhido e de 'RUA ARGENTINA DE OLIVEIRA FERREIRA 185, 185, FERTIZA' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G251" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>220557927</t>
+        </is>
+      </c>
+      <c r="B252" t="n">
+        <v>932</v>
+      </c>
+      <c r="C252" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.6074363,-46.9452363,3a,75y,18.38h,112.86t/data=!3m7!1e1!3m5!1sAlwiceZ_aak1TnVuIgMutw!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-22.86322483808398%26panoid%3DAlwiceZ_aak1TnVuIgMutw%26yaw%3D18.384725296474638!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>RUA ARGENTINA DE OLIVEIRA FERREIRA 195, 195, FERTIZA</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (2.5m, 66 graus) e rumo (33.0m, 33 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G252" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>1347586020</t>
+        </is>
+      </c>
+      <c r="B253" t="n">
+        <v>933</v>
+      </c>
+      <c r="C253" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.607624,-46.9451899,3a,90y,86.01h,124.28t/data=!3m7!1e1!3m5!1scsy6fhecN-LQfoAN_eCBlQ!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-34.27506963149922%26panoid%3Dcsy6fhecN-LQfoAN_eCBlQ%26yaw%3D86.01096705794882!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>RUA ARGENTINA DE OLIVEIRA FERREIRA 215, 215, FERTIZA</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (6.7m, 94 graus) e rumo (39.6m, 83 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G253" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>224052795</t>
+        </is>
+      </c>
+      <c r="B254" t="n">
+        <v>935</v>
+      </c>
+      <c r="C254" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.6081323,-46.9450663,3a,75y,119.78h,108.43t/data=!3m7!1e1!3m5!1sxJQF98o3RX6H5JKuNOenPQ!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-18.433076064584952%26panoid%3DxJQF98o3RX6H5JKuNOenPQ%26yaw%3D119.77856328574163!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>RUA ARGENTINA DE OLIVEIRA FERREIRA 222, 222, FERTIZA</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (12.7m, 54 graus) e rumo (59.9m, 46 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G254" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>221621822</t>
+        </is>
+      </c>
+      <c r="B255" t="n">
+        <v>937</v>
+      </c>
+      <c r="C255" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.6089772,-46.9448798,3a,90y,90.49h,118.38t/data=!3m7!1e1!3m5!1sVjzPmYfJmWeJpPcPPy4PSQ!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-28.38151710004908%26panoid%3DVjzPmYfJmWeJpPcPPy4PSQ%26yaw%3D90.49029181867172!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>RUA ARGENTINA DE OLIVEIRA FERREIRA 335, 335, FERTIZA</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>confirmar - poste mais proximo (4.3m) tem 80 graus de diferenca de rumo, mas esta perto o suficiente pra ser so ruido de GPS</t>
+        </is>
+      </c>
+      <c r="G255" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>350236641</t>
+        </is>
+      </c>
+      <c r="B256" t="n">
+        <v>941</v>
+      </c>
+      <c r="C256" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.6067405,-46.9446374,3a,48.9y,221.09h,108.41t/data=!3m7!1e1!3m5!1sAtq1trS_BuJNA9XSbVVX3w!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-18.41094448425467%26panoid%3DAtq1trS_BuJNA9XSbVVX3w%26yaw%3D221.09256553957786!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>RUA JOAQUIM TEODORO DA SILVA 371, 371, FERTIZA</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>confirmar - poste mais proximo (8.9m) tem 103 graus de diferenca de rumo, mas esta perto o suficiente pra ser so ruido de GPS</t>
+        </is>
+      </c>
+      <c r="G256" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>220853314</t>
+        </is>
+      </c>
+      <c r="B257" t="n">
+        <v>945</v>
+      </c>
+      <c r="C257" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.6063386,-46.944529,3a,90y,71.42h,131.27t/data=!3m7!1e1!3m5!1sOlC7GAlt1ALC2JjO1fv5nw!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-41.26570330431224%26panoid%3DOlC7GAlt1ALC2JjO1fv5nw%26yaw%3D71.41896557246031!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>RUA DONA ADELIA LELIS 110, 110, FERTIZA</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (6.8m, 94 graus) e rumo (42.6m, 76 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G257" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>219991785</t>
+        </is>
+      </c>
+      <c r="B258" t="n">
+        <v>946</v>
+      </c>
+      <c r="C258" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.6060548,-46.944526,3a,90y,30.17h,115.16t/data=!3m7!1e1!3m5!1sRmtyzxo2-mJ9thNWx9iXxg!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-25.163421652126033%26panoid%3DRmtyzxo2-mJ9thNWx9iXxg%26yaw%3D30.171519297266798!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>RUA DONA ADELIA LELIS 70, 70, FERTIZA</t>
+        </is>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (11.5m, 48 graus) e rumo (43.1m, 33 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G258" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>221621844</t>
+        </is>
+      </c>
+      <c r="B259" t="n">
+        <v>947</v>
+      </c>
+      <c r="C259" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.6057745,-46.9445327,3a,75y,35.16h,117.27t/data=!3m7!1e1!3m5!1s_qKnSh0h78HTF2ZkW12Qnw!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-27.26692794979992%26panoid%3D_qKnSh0h78HTF2ZkW12Qnw%26yaw%3D35.16155911478792!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>RUA DONA ADELIA LELIS 21, 21, FERTIZA</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (12.0m, 42 graus) e rumo (55.2m, 15 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G259" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>223323829</t>
+        </is>
+      </c>
+      <c r="B260" t="n">
+        <v>949</v>
+      </c>
+      <c r="C260" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.6053067,-46.9443275,3a,90y,22.39h,129.22t/data=!3m7!1e1!3m5!1s4NjMaD0883Fz96LfWlS94g!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-39.223200477330096%26panoid%3D4NjMaD0883Fz96LfWlS94g%26yaw%3D22.385615172339836!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>RUA DONATO PINHEIRO DOS SANTOS 448, 448, JOAO RIBEIRO</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (2.5m, 117 graus) e rumo (61.5m, 57 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G260" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>219991916</t>
+        </is>
+      </c>
+      <c r="B261" t="n">
+        <v>958</v>
+      </c>
+      <c r="C261" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.6139245,-46.9464096,3a,75y,31.67h,108.62t/data=!3m7!1e1!3m5!1sB-Z1gJ7vfVR1ngnyjN-hRw!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-18.615185329723815%26panoid%3DB-Z1gJ7vfVR1ngnyjN-hRw%26yaw%3D31.666376753971203!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>RUA ZEQUINHA GOULART 175, 175, FERTIZA</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>ATENCAO nome de rua muito diferente: Street View diz o endereco e '232 R. José da Cunha Júnior', cod_id escolhido e de 'RUA ZEQUINHA GOULART 175, 175, FERTIZA' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G261" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>223976782</t>
+        </is>
+      </c>
+      <c r="B262" t="n">
+        <v>959</v>
+      </c>
+      <c r="C262" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.6137636,-46.9460031,3a,75y,291.46h,107.2t/data=!3m7!1e1!3m5!1sZLnJW8wl93htkQrKQGRB5A!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-17.20090180782813%26panoid%3DZLnJW8wl93htkQrKQGRB5A%26yaw%3D291.4610624012514!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>RUA ZEQUINHA GOULART 30, 30, FERTIZA</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (13.8m, 26 graus) e rumo (57.3m, 10 graus) nao concordam com confianca; ATENCAO nome de rua muito diferente: Street View diz o endereco e '2315 Av. Geraldo Porfírio Botelho', cod_id escolhido e de 'RUA ZEQUINHA GOULART 30, 30, FERTIZA' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G262" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>223390210</t>
+        </is>
+      </c>
+      <c r="B263" t="n">
+        <v>960</v>
+      </c>
+      <c r="C263" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.6136685,-46.9458179,3a,75y,5.27h,107.65t/data=!3m7!1e1!3m5!1sPdY0lsA-7-3Tf1uhX-LKUQ!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-17.64548610137723%26panoid%3DPdY0lsA-7-3Tf1uhX-LKUQ%26yaw%3D5.266791312091003!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>RUA ZEQUINHA GOULART 30, 30, FERTIZA</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>ATENCAO nome de rua muito diferente: Street View diz o endereco e '464 Av. Geraldo Porfírio Botelho', cod_id escolhido e de 'RUA ZEQUINHA GOULART 30, 30, FERTIZA' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G263" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>223390145</t>
+        </is>
+      </c>
+      <c r="B264" t="n">
+        <v>961</v>
+      </c>
+      <c r="C264" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.6134845,-46.945493,3a,75y,328.76h,116.93t/data=!3m7!1e1!3m5!1siMHOFVuaILJEwQI7aJHWNg!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-26.928831949289318%26panoid%3DiMHOFVuaILJEwQI7aJHWNg%26yaw%3D328.76468596386417!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>RUA ARIOVALDO AFONSO 730, 730, FERTIZA</t>
+        </is>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>ATENCAO nome de rua muito diferente: Street View diz o endereco e '2265 Av. Geraldo Porfírio Botelho', cod_id escolhido e de 'RUA ARIOVALDO AFONSO 730, 730, FERTIZA' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G264" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>223976726</t>
+        </is>
+      </c>
+      <c r="B265" t="n">
+        <v>963</v>
+      </c>
+      <c r="C265" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.6132231,-46.94499,3a,75y,341.91h,116.82t/data=!3m7!1e1!3m5!1sjLdvtyL2VRWDABu1Y4x1xw!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-26.81664059045997%26panoid%3DjLdvtyL2VRWDABu1Y4x1xw%26yaw%3D341.90906913303064!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>BENEDITO REZENDE 2340, 2340, FERTIZA</t>
+        </is>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>ATENCAO nome de rua muito diferente: Street View diz o endereco e '2215 Av. Geraldo Porfírio Botelho', cod_id escolhido e de 'BENEDITO REZENDE 2340, 2340, FERTIZA' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G265" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>223976723</t>
+        </is>
+      </c>
+      <c r="B266" t="n">
+        <v>966</v>
+      </c>
+      <c r="C266" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.6127268,-46.9448576,3a,90y,100.53h,124.94t/data=!3m7!1e1!3m5!1sBBGDqIaiCidJcac4RLEbVA!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-34.944804310831586%26panoid%3DBBGDqIaiCidJcac4RLEbVA%26yaw%3D100.5324073147426!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>RUA BENEDITO REZENDE 819, 819, FERTIZA</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (2.4m, 169 graus) e rumo (29.6m, 63 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G266" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>219298139</t>
+        </is>
+      </c>
+      <c r="B267" t="n">
+        <v>970</v>
+      </c>
+      <c r="C267" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.6129022,-46.9443835,3a,55.4y,309.19h,110.81t/data=!3m7!1e1!3m5!1slSb2H9-cqlfLGM5zrY9qYg!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-20.814626459652217%26panoid%3DlSb2H9-cqlfLGM5zrY9qYg%26yaw%3D309.1921520177069!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>RUA BENEDITO REZENDE 819, 819, FERTIZA</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>ATENCAO nome de rua muito diferente: Street View diz o endereco e '2165 Av. Geraldo Porfírio Botelho', cod_id escolhido e de 'RUA BENEDITO REZENDE 819, 819, FERTIZA' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G267" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>219991903</t>
+        </is>
+      </c>
+      <c r="B268" t="n">
+        <v>971</v>
+      </c>
+      <c r="C268" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.6127635,-46.9441087,3a,75y,307.7h,111.6t/data=!3m7!1e1!3m5!1sHkNLzekbzCl4ncCKCAVksw!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-21.60277093377094%26panoid%3DHkNLzekbzCl4ncCKCAVksw%26yaw%3D307.69987095101135!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>RUA GASTAO SANTOS 225, 225, FERTIZA</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (13.8m, 6 graus) e rumo (61.5m, 3 graus) nao concordam com confianca; ATENCAO nome de rua muito diferente: Street View diz o endereco e '2165 Av. Geraldo Porfírio Botelho', cod_id escolhido e de 'RUA GASTAO SANTOS 225, 225, FERTIZA' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G268" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>220780133</t>
+        </is>
+      </c>
+      <c r="B269" t="n">
+        <v>972</v>
+      </c>
+      <c r="C269" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.6126276,-46.9438457,3a,48.9y,295.03h,103.9t/data=!3m7!1e1!3m5!1sPgutPhZSnMjNzsF9_n3e0Q!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-13.89654565618794%26panoid%3DPgutPhZSnMjNzsF9_n3e0Q%26yaw%3D295.0332047245622!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>RUA GASTAO SANTOS 225, 225, FERTIZA</t>
+        </is>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>ATENCAO nome de rua muito diferente: Street View diz o endereco e '2057 Av. Geraldo Porfírio Botelho', cod_id escolhido e de 'RUA GASTAO SANTOS 225, 225, FERTIZA' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G269" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>601456298</t>
+        </is>
+      </c>
+      <c r="B270" t="n">
+        <v>991</v>
+      </c>
+      <c r="C270" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.6116421,-46.9423169,3a,75y,293.13h,107.42t/data=!3m7!1e1!3m5!1sZajLlsNdP1OR01TzrTtF7g!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-17.41611211962845%26panoid%3DZajLlsNdP1OR01TzrTtF7g%26yaw%3D293.1306639933246!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>AVENIDA GERALDO PORFIRIO BOTELHO 1960, 1960, FERTIZA</t>
+        </is>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>ATENCAO nome de rua muito diferente: Street View diz o endereco e '131 R. José da Cruz', cod_id escolhido e de 'AVENIDA GERALDO PORFIRIO BOTELHO 1960, 1960, FERTIZA' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G270" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>601456297</t>
+        </is>
+      </c>
+      <c r="B271" t="n">
+        <v>992</v>
+      </c>
+      <c r="C271" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.6114395,-46.9426707,3a,75y,266.13h,110.22t/data=!3m7!1e1!3m5!1sL0uSLbRJ6ffIS5w_lUETOw!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-20.220856600783236%26panoid%3DL0uSLbRJ6ffIS5w_lUETOw%26yaw%3D266.1274597225245!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>AVENIDA PREFEITO ARACELY DE PAULA 370, 370, FERTIZA</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>ATENCAO nome de rua muito diferente: Street View diz o endereco e '131 R. José da Cruz', cod_id escolhido e de 'AVENIDA PREFEITO ARACELY DE PAULA 370, 370, FERTIZA' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G271" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>601456294</t>
+        </is>
+      </c>
+      <c r="B272" t="n">
+        <v>993</v>
+      </c>
+      <c r="C272" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.6112543,-46.9430874,3a,90y,221.3h,118.12t/data=!3m7!1e1!3m5!1saWDBubRgzyj_jp4yEHHQew!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-28.117130114656902%26panoid%3DaWDBubRgzyj_jp4yEHHQew%26yaw%3D221.29795017430132!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>AVENIDA PREFEITO ARACELY DE PAULA 405, 405, FERTIZA</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (4.2m, 166 graus) e rumo (32.7m, 38 graus) nao concordam com confianca; ATENCAO nome de rua muito diferente: Street View diz o endereco e '1 R. José da Cruz', cod_id escolhido e de 'AVENIDA PREFEITO ARACELY DE PAULA 405, 405, FERTIZA' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G272" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>220780134</t>
+        </is>
+      </c>
+      <c r="B273" t="n">
+        <v>1011</v>
+      </c>
+      <c r="C273" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.6110839,-46.9452534,3a,90y,87.78h,126.54t/data=!3m7!1e1!3m5!1sdw7IRLXrrwIezSe1GZO5pA!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-36.538203928303616%26panoid%3Ddw7IRLXrrwIezSe1GZO5pA%26yaw%3D87.77624240059495!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>RUA BENEDITO REZENDE 545, 545, FERTIZA</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (1.6m, 81 graus) e rumo (40.2m, 69 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G273" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>222494485</t>
+        </is>
+      </c>
+      <c r="B274" t="n">
+        <v>1012</v>
+      </c>
+      <c r="C274" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.6107715,-46.9453286,3a,90y,69.57h,126.11t/data=!3m7!1e1!3m5!1sCMmjGTj1KIXDlBnMdgI8ig!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-36.111896882247805%26panoid%3DCMmjGTj1KIXDlBnMdgI8ig%26yaw%3D69.56849887228579!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>RUA ANTONIO BARRETO 490, 490, FERTIZA</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>confirmar - poste mais proximo (2.0m) tem 80 graus de diferenca de rumo, mas esta perto o suficiente pra ser so ruido de GPS; ATENCAO nome de rua muito diferente: Street View diz o endereco e '88 R. Benedito Rezende', cod_id escolhido e de 'RUA ANTONIO BARRETO 490, 490, FERTIZA' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G274" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>350236578</t>
+        </is>
+      </c>
+      <c r="B275" t="n">
+        <v>1019</v>
+      </c>
+      <c r="C275" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.6100655,-46.9456212,3a,90y,19.58h,116.17t/data=!3m7!1e1!3m5!1sx11Ez74MtbFqDCXfPar1XQ!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-26.171664213937845%26panoid%3Dx11Ez74MtbFqDCXfPar1XQ%26yaw%3D19.58402806374983!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>RUA SELDA DE CASTRO ALVES 486, 486, FERTIZA</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (14.3m, 46 graus) e rumo (17.8m, 12 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G275" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>219991187</t>
+        </is>
+      </c>
+      <c r="B276" t="n">
+        <v>1027</v>
+      </c>
+      <c r="C276" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.6103298,-46.9445487,3a,75y,104.36h,118.19t/data=!3m7!1e1!3m5!1saw1wVBY2aFrscvIktGOC2w!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-28.189011681042288%26panoid%3Daw1wVBY2aFrscvIktGOC2w%26yaw%3D104.36436345011532!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>RUA ARGENTINA DE OLIVEIRA FERREIRA 467, 467, FERTIZA</t>
+        </is>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (3.2m, 97 graus) e rumo (28.2m, 59 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G276" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>220853357</t>
+        </is>
+      </c>
+      <c r="B277" t="n">
+        <v>1043</v>
+      </c>
+      <c r="C277" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.6105636,-46.9427034,3a,90y,73.25h,122.9t/data=!3m7!1e1!3m5!1sgI7EqkZEqlWFskvhq_UAgg!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-32.90206096467773%26panoid%3DgI7EqkZEqlWFskvhq_UAgg%26yaw%3D73.25262786357017!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>RUA JOSE BARBOSA DE CASTRO 535, 535, FERTIZA</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (7.3m, 53 graus) e rumo (37.5m, 32 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G277" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>222496779</t>
+        </is>
+      </c>
+      <c r="B278" t="n">
+        <v>1048</v>
+      </c>
+      <c r="C278" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.6107082,-46.9435516,3a,90y,109.98h,129.91t/data=!3m7!1e1!3m5!1s42ji24p7c8a8NI0kAeL-zA!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-39.910506990143176%26panoid%3D42ji24p7c8a8NI0kAeL-zA%26yaw%3D109.98066296932596!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>RUA DONA ADELIA LELIS 595, 595, FERTIZA</t>
+        </is>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (4.2m, 67 graus) e rumo (37.2m, 48 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G278" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>738920114</t>
+        </is>
+      </c>
+      <c r="B279" t="n">
+        <v>1059</v>
+      </c>
+      <c r="C279" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.6103499,-46.9419572,3a,90y,288.82h,130.32t/data=!3m7!1e1!3m5!1sPUrkyFGnjvVdtKj-fvaVKA!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-40.32356767419461%26panoid%3DPUrkyFGnjvVdtKj-fvaVKA%26yaw%3D288.81691480179404!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>AVENIDA PREFEITO ARACELY DE PAULA 175, 175, FERTIZA</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (8.3m, 156 graus) e rumo (24.1m, 45 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G279" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>219385332</t>
+        </is>
+      </c>
+      <c r="B280" t="n">
+        <v>1071</v>
+      </c>
+      <c r="C280" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.590787,-46.9347562,3a,49.7y,20.33h,101.36t/data=!3m7!1e1!3m5!1sX3e20EaCqHRIOtHIcKl9wg!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-11.36339127175593%26panoid%3DX3e20EaCqHRIOtHIcKl9wg%26yaw%3D20.330287771074214!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>RUA TEREZINHA NATAL CONTATO 55, 55, CENTRO</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (10.0m, 16 graus) e rumo (41.2m, 12 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G280" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>221704482</t>
+        </is>
+      </c>
+      <c r="B281" t="n">
+        <v>1075</v>
+      </c>
+      <c r="C281" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5913187,-46.9349518,3a,90y,42h,125.75t/data=!3m7!1e1!3m5!1sFYS8VNKzBGkvsRXiODHMDQ!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-35.751561357028706%26panoid%3DFYS8VNKzBGkvsRXiODHMDQ%26yaw%3D42.00047263773909!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>RUA PEPURURE 140, 140, CENTRO</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (1.6m, 128 graus) e rumo (42.3m, 39 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G281" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>220854166</t>
+        </is>
+      </c>
+      <c r="B282" t="n">
+        <v>1077</v>
+      </c>
+      <c r="C282" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5916337,-46.9345123,3a,90y,20.04h,117.79t/data=!3m7!1e1!3m5!1srojGdYZaChXL00eCMdsv0Q!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-27.787148361964142%26panoid%3DrojGdYZaChXL00eCMdsv0Q%26yaw%3D20.037075823542832!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>RUA PEPURURE 217, 217, CENTRO</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (0.6m, 171 graus) e rumo (59.2m, 74 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G282" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>223455916</t>
+        </is>
+      </c>
+      <c r="B283" t="n">
+        <v>1079</v>
+      </c>
+      <c r="C283" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5919524,-46.9339959,3a,75y,150.39h,122.48t/data=!3m7!1e1!3m5!1sIm5ewG9yIbPGnJqz4M2_BQ!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-32.478691772241376%26panoid%3DIm5ewG9yIbPGnJqz4M2_BQ%26yaw%3D150.38978089584793!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>RUA PEPURURE 287, 287, CENTRO</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>ATENCAO nome de rua muito diferente: Street View diz o endereco e '172 R. Cecílio Salomão', cod_id escolhido e de 'RUA PEPURURE 287, 287, CENTRO' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G283" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>224358070</t>
+        </is>
+      </c>
+      <c r="B284" t="n">
+        <v>1082</v>
+      </c>
+      <c r="C284" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5921959,-46.9337987,3a,75y,46.61h,119.12t/data=!3m7!1e1!3m5!1s6XoSjbzypVTlnb4ZNMrIJw!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-29.118109906055764%26panoid%3D6XoSjbzypVTlnb4ZNMrIJw%26yaw%3D46.61054004281236!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>RUA PEPURURE 307, 307, CENTRO</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (1.3m, 52 graus) e rumo (43.2m, 51 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G284" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>219385333</t>
+        </is>
+      </c>
+      <c r="B285" t="n">
+        <v>1083</v>
+      </c>
+      <c r="C285" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5924268,-46.9336274,3a,90y,60.18h,130.75t/data=!3m7!1e1!3m5!1sACG94WYbrz4-uvG2wnrdBw!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-40.754366759053966%26panoid%3DACG94WYbrz4-uvG2wnrdBw%26yaw%3D60.17941423407531!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>RUA PEPURURE 307, 307, CENTRO</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (3.3m, 76 graus) e rumo (67.5m, 58 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>219992743</t>
+        </is>
+      </c>
+      <c r="B286" t="n">
+        <v>1084</v>
+      </c>
+      <c r="C286" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5926618,-46.9334768,3a,90y,51.38h,130.83t/data=!3m7!1e1!3m5!1sRNYXh0m-F_0gVY2bUDXnMA!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-40.83463514514105%26panoid%3DRNYXh0m-F_0gVY2bUDXnMA%26yaw%3D51.38144472502934!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>RUA PEPURURE 330, 330, CENTRO</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>confirmar - poste mais proximo (1.4m) tem 96 graus de diferenca de rumo, mas esta perto o suficiente pra ser so ruido de GPS</t>
+        </is>
+      </c>
+      <c r="G286" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>224358122</t>
+        </is>
+      </c>
+      <c r="B287" t="n">
+        <v>1086</v>
+      </c>
+      <c r="C287" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5918191,-46.9349608,3a,90y,314.63h,119.52t/data=!3m7!1e1!3m5!1sa6OFE5KB1sIuFnKf9xF3Ig!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-29.51938066986048%26panoid%3Da6OFE5KB1sIuFnKf9xF3Ig%26yaw%3D314.6336486063422!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>TRAVESSA SANTA ISABEL 91, 91, CENTRO</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (6.3m, 49 graus) e rumo (55.7m, 45 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G287" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>223978099</t>
+        </is>
+      </c>
+      <c r="B288" t="n">
+        <v>1087</v>
+      </c>
+      <c r="C288" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5917229,-46.9337928,3a,90y,177.37h,112.11t/data=!3m7!1e1!3m5!1sziJWiuMHHVefOMohhhaUHg!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-22.109424822499918%26panoid%3DziJWiuMHHVefOMohhhaUHg%26yaw%3D177.36648825883637!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>RUA CECILIO SALOMAO 200, 200, CENTRO</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (10.3m, 24 graus) e rumo (52.8m, 2 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G288" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>222733206</t>
+        </is>
+      </c>
+      <c r="B289" t="n">
+        <v>1091</v>
+      </c>
+      <c r="C289" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5909752,-46.9333076,3a,73.9y,261.1h,133.22t/data=!3m7!1e1!3m5!1s-RBlvbdDw-jEdsDrf_-yOg!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-43.22171996292664%26panoid%3D-RBlvbdDw-jEdsDrf_-yOg%26yaw%3D261.1047096619453!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>RUA CECILIO SALOMAO 975, 975, CENTRO</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>ATENCAO nome de rua muito diferente: Street View diz o endereco e '977 Av. Dâmaso Drumond', cod_id escolhido e de 'RUA CECILIO SALOMAO 975, 975, CENTRO' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G289" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>223978091</t>
+        </is>
+      </c>
+      <c r="B290" t="n">
+        <v>1093</v>
+      </c>
+      <c r="C290" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5909625,-46.9354067,3a,90y,345.92h,123.69t/data=!3m7!1e1!3m5!1sNydTA1tCs-oaQnNJBWiuIg!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-33.6879101127781%26panoid%3DNydTA1tCs-oaQnNJBWiuIg%26yaw%3D345.91874832443204!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>RUA PEPURURE 110, 110, CENTRO</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (8.1m, 52 graus) e rumo (46.5m, 41 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G290" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>223455871</t>
+        </is>
+      </c>
+      <c r="B291" t="n">
+        <v>1094</v>
+      </c>
+      <c r="C291" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5907248,-46.9357197,3a,90y,0.36h,139.49t/data=!3m7!1e1!3m5!1sFQZP_mIZEaX-PCaSUMXnrQ!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-49.49136505576715%26panoid%3DFQZP_mIZEaX-PCaSUMXnrQ%26yaw%3D0.3629594361283761!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>RUA LIMIRIO AFONSO 157, 157, CENTRO</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (5.3m, 87 graus) e rumo (59.2m, 54 graus) nao concordam com confianca; ATENCAO nome de rua muito diferente: Street View diz o endereco e '73 R. Pepurure', cod_id escolhido e de 'RUA LIMIRIO AFONSO 157, 157, CENTRO' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G291" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>222495160</t>
+        </is>
+      </c>
+      <c r="B292" t="n">
+        <v>1095</v>
+      </c>
+      <c r="C292" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5905397,-46.9359728,3a,75y,329.84h,118.71t/data=!3m7!1e1!3m5!1sr-gA0Npuvkcf4DybXi5rYA!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-28.710879956717008%26panoid%3Dr-gA0Npuvkcf4DybXi5rYA%26yaw%3D329.83861939675757!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>RUA PEPURURE 22, 22, CENTRO</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>confirmar - poste mais proximo (2.7m) tem 80 graus de diferenca de rumo, mas esta perto o suficiente pra ser so ruido de GPS</t>
+        </is>
+      </c>
+      <c r="G292" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>224358032</t>
+        </is>
+      </c>
+      <c r="B293" t="n">
+        <v>1096</v>
+      </c>
+      <c r="C293" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5903562,-46.9362198,3a,75y,72.9h,128.04t/data=!3m7!1e1!3m5!1sy83nJQwyL-HVZcisKCUWiA!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-38.0405605240573%26panoid%3Dy83nJQwyL-HVZcisKCUWiA%26yaw%3D72.89666023108619!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>RUA PEPURURE 12, 12, CENTRO</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (7.6m, 70 graus) e rumo (31.6m, 59 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G293" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>220854077</t>
+        </is>
+      </c>
+      <c r="B294" t="n">
+        <v>1097</v>
+      </c>
+      <c r="C294" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5902005,-46.9362475,3a,48.9y,224.1h,115.28t/data=!3m7!1e1!3m5!1sCaPsylHiN5vsjPrJAn6aGw!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-25.277960419800436%26panoid%3DCaPsylHiN5vsjPrJAn6aGw%26yaw%3D224.0969465458949!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>RUA HERCULANO BATISTA 146, 146, CENTRO</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>ATENCAO nome de rua muito diferente: Street View diz o endereco e '127 R. Santa Rita', cod_id escolhido e de 'RUA HERCULANO BATISTA 146, 146, CENTRO' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G294" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>223977756</t>
+        </is>
+      </c>
+      <c r="B295" t="n">
+        <v>1102</v>
+      </c>
+      <c r="C295" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5886602,-46.9368364,3a,73.9y,158.72h,116.3t/data=!3m7!1e1!3m5!1sTXHWycv9r5I7D26vM9OcIg!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-26.29567934544214%26panoid%3DTXHWycv9r5I7D26vM9OcIg%26yaw%3D158.7224865422628!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>RUA ALEXANDRE GONDIM 240, 240, CENTRO</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>ATENCAO nome de rua muito diferente: Street View diz o endereco e '85 Tv. Zéca Montandon', cod_id escolhido e de 'RUA ALEXANDRE GONDIM 240, 240, CENTRO' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G295" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>221986648</t>
+        </is>
+      </c>
+      <c r="B296" t="n">
+        <v>1106</v>
+      </c>
+      <c r="C296" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5893972,-46.9379758,3a,90y,7.93h,124.01t/data=!3m7!1e1!3m5!1sxrPYjtgHcf17cLPL--DGhw!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-34.01274812048875%26panoid%3DxrPYjtgHcf17cLPL--DGhw%26yaw%3D7.927110683342447!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>PRACA CORONEL JOSE ADOLFO 15, 15, CENTRO</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>confirmar - poste mais proximo (4.1m) tem 171 graus de diferenca de rumo, mas esta perto o suficiente pra ser so ruido de GPS</t>
+        </is>
+      </c>
+      <c r="G296" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>219384947</t>
+        </is>
+      </c>
+      <c r="B297" t="n">
+        <v>1109</v>
+      </c>
+      <c r="C297" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.588635,-46.9363427,3a,75y,273.45h,140.55t/data=!3m7!1e1!3m5!1sZknXMnKLg6zGLx_T0RC0GA!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-50.54540153449025%26panoid%3DZknXMnKLg6zGLx_T0RC0GA%26yaw%3D273.45165246987193!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>RUA ALEXANDRE GONDIM 157, 157, CENTRO</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (14.3m, 8 graus) e rumo (68.2m, 3 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G297" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>224357718</t>
+        </is>
+      </c>
+      <c r="B298" t="n">
+        <v>1110</v>
+      </c>
+      <c r="C298" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5886118,-46.9359528,3a,75y,284h,119.42t/data=!3m7!1e1!3m5!1seLrXMTlEOmkaoFxEhLegdA!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-29.4219541801761%26panoid%3DeLrXMTlEOmkaoFxEhLegdA%26yaw%3D283.996101096886!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>RUA ALEXANDRE GONDIM 209, 209, CENTRO</t>
+        </is>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (15.2m, 19 graus) e rumo (55.2m, 18 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G298" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>219992912</t>
+        </is>
+      </c>
+      <c r="B299" t="n">
+        <v>1112</v>
+      </c>
+      <c r="C299" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5885786,-46.9354716,3a,75y,60.11h,113.35t/data=!3m7!1e1!3m5!1s18xAsSiQraMflEPVKgqdZg!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-23.3505150301189%26panoid%3D18xAsSiQraMflEPVKgqdZg%26yaw%3D60.10817547460569!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>RUA ALEXANDRE GONDIM 267, 267, CENTRO</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>confirmar - poste mais proximo (0.8m) tem 89 graus de diferenca de rumo, mas esta perto o suficiente pra ser so ruido de GPS</t>
+        </is>
+      </c>
+      <c r="G299" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>219385325</t>
+        </is>
+      </c>
+      <c r="B300" t="n">
+        <v>1114</v>
+      </c>
+      <c r="C300" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5885936,-46.9347644,3a,90y,21.69h,115.45t/data=!3m7!1e1!3m5!1sIfeDYxA2p9lXvMOejnyQ7g!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-25.449002195587653%26panoid%3DIfeDYxA2p9lXvMOejnyQ7g%26yaw%3D21.692641453590706!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>RUA ITACURU 551, 551, CENTRO</t>
+        </is>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (6.4m, 70 graus) e rumo (47.3m, 44 graus) nao concordam com confianca; ATENCAO nome de rua muito diferente: Street View diz o endereco e '454 R. Alexandre Gondin', cod_id escolhido e de 'RUA ITACURU 551, 551, CENTRO' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G300" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>222495162</t>
+        </is>
+      </c>
+      <c r="B301" t="n">
+        <v>1120</v>
+      </c>
+      <c r="C301" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5905388,-46.9364134,3a,75y,230.27h,118.11t/data=!3m7!1e1!3m5!1sNfbSeuQCsMRwGq-j9lFbeQ!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-28.106381025753194%26panoid%3DNfbSeuQCsMRwGq-j9lFbeQ%26yaw%3D230.27181294891207!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>RUA SANTA RITA 89, 89, CENTRO</t>
+        </is>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>confirmar - poste mais proximo (5.5m) tem 80 graus de diferenca de rumo, mas esta perto o suficiente pra ser so ruido de GPS</t>
+        </is>
+      </c>
+      <c r="G301" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>221704411</t>
+        </is>
+      </c>
+      <c r="B302" t="n">
+        <v>1121</v>
+      </c>
+      <c r="C302" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5908036,-46.93655,3a,90y,257.47h,129.64t/data=!3m7!1e1!3m5!1slkZ9KsDlm5F5vT1zCMUSRQ!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-39.63884232026871%26panoid%3DlkZ9KsDlm5F5vT1zCMUSRQ%26yaw%3D257.4686726030663!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>RUA SANTA RITA 71, 71, CENTRO</t>
+        </is>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>confirmar - poste mais proximo (6.5m) tem 63 graus de diferenca de rumo, mas esta perto o suficiente pra ser so ruido de GPS</t>
+        </is>
+      </c>
+      <c r="G302" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>220854032</t>
+        </is>
+      </c>
+      <c r="B303" t="n">
+        <v>1129</v>
+      </c>
+      <c r="C303" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5922487,-46.9375212,3a,90y,324.53h,123.07t/data=!3m7!1e1!3m5!1s8-bvEQrggMLtsWt_it-TCA!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-33.07353668359636%26panoid%3D8-bvEQrggMLtsWt_it-TCA%26yaw%3D324.5303415993376!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>RUA MARIANO DE AVILA 106, 106, CENTRO</t>
+        </is>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (7.2m, 61 graus) e rumo (35.1m, 49 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G303" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>219992875</t>
+        </is>
+      </c>
+      <c r="B304" t="n">
+        <v>1132</v>
+      </c>
+      <c r="C304" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5928019,-46.9380459,3a,90y,347.07h,119.52t/data=!3m7!1e1!3m5!1s3N0TWIs6XEsYiFW2VnktyA!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-29.523018571244734%26panoid%3D3N0TWIs6XEsYiFW2VnktyA%26yaw%3D347.07046802027673!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>RUA MARIANO DE AVILA 170, 170, CENTRO</t>
+        </is>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>confirmar - poste mais proximo (4.9m) tem 65 graus de diferenca de rumo, mas esta perto o suficiente pra ser so ruido de GPS</t>
+        </is>
+      </c>
+      <c r="G304" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>223455553</t>
+        </is>
+      </c>
+      <c r="B305" t="n">
+        <v>1133</v>
+      </c>
+      <c r="C305" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5929901,-46.9382279,3a,90y,265.99h,143.41t/data=!3m7!1e1!3m5!1s9REYNEtNMadJ6jn8wKxZSQ!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-53.40886895136239%26panoid%3D9REYNEtNMadJ6jn8wKxZSQ%26yaw%3D265.9942979613418!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>RUA MARIANO DE AVILA 222, 222, CENTRO</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (13.6m, 32 graus) e rumo (32.3m, 4 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G305" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>222494815</t>
+        </is>
+      </c>
+      <c r="B306" t="n">
+        <v>1139</v>
+      </c>
+      <c r="C306" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5941084,-46.9392673,3a,48.9y,246.66h,113.96t/data=!3m7!1e1!3m5!1sR_mQFK5I8SyM1XEBuYD92Q!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-23.96328484147466%26panoid%3DR_mQFK5I8SyM1XEBuYD92Q%26yaw%3D246.65914597743858!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>AVENIDA GETULIO VARGAS 0, 0, CENTRO</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>ATENCAO nome de rua muito diferente: Street View diz o endereco e '388 R. Mariano de Ávila', cod_id escolhido e de 'AVENIDA GETULIO VARGAS 0, 0, CENTRO' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G306" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>221704219</t>
+        </is>
+      </c>
+      <c r="B307" t="n">
+        <v>1143</v>
+      </c>
+      <c r="C307" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5948761,-46.9399925,3a,48.9y,245.49h,111.49t/data=!3m7!1e1!3m5!1sUYzSIUnITfDlcepmlkS78w!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-21.494544848400807%26panoid%3DUYzSIUnITfDlcepmlkS78w%26yaw%3D245.49417411052923!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>RUA DOM BOSCO 0, 0, CENTRO</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>ATENCAO nome de rua muito diferente: Street View diz o endereco e '74 R. Mariano de Ávila', cod_id escolhido e de 'RUA DOM BOSCO 0, 0, CENTRO' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G307" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>219992900</t>
+        </is>
+      </c>
+      <c r="B308" t="n">
+        <v>1146</v>
+      </c>
+      <c r="C308" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5897814,-46.9374621,3a,90y,76.46h,134.66t/data=!3m7!1e1!3m5!1skBdqMy2ObugoSBN_XSGUqA!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-44.65542014658715%26panoid%3DkBdqMy2ObugoSBN_XSGUqA%26yaw%3D76.46198556157094!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>RUA CONEGO CASSIANO 81, 81, CENTRO</t>
+        </is>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>confirmar - poste mais proximo (2.3m) tem 169 graus de diferenca de rumo, mas esta perto o suficiente pra ser so ruido de GPS</t>
+        </is>
+      </c>
+      <c r="G308" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>223455533</t>
+        </is>
+      </c>
+      <c r="B309" t="n">
+        <v>1148</v>
+      </c>
+      <c r="C309" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.590252,-46.9371021,3a,90y,6.16h,115.33t/data=!3m7!1e1!3m5!1s9K6wWemWVkegEDC9UcuCuA!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-25.33070175601607%26panoid%3D9K6wWemWVkegEDC9UcuCuA%26yaw%3D6.159296477714545!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>RUA CONEGO CASSIANO 155, 155, CENTRO</t>
+        </is>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (5.1m, 51 graus) e rumo (35.6m, 39 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G309" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>223977738</t>
+        </is>
+      </c>
+      <c r="B310" t="n">
+        <v>1149</v>
+      </c>
+      <c r="C310" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5904157,-46.936999,3a,90y,98.23h,119.7t/data=!3m7!1e1!3m5!1s7tXWpUjqB9bH8O6An4Hdwg!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-29.70149939332461%26panoid%3D7tXWpUjqB9bH8O6An4Hdwg%26yaw%3D98.226405496421!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>RUA CONEGO CASSIANO 164, 164, CENTRO</t>
+        </is>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (2.2m, 131 graus) e rumo (54.1m, 52 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G310" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>219384901</t>
+        </is>
+      </c>
+      <c r="B311" t="n">
+        <v>1150</v>
+      </c>
+      <c r="C311" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5906534,-46.936867,3a,90y,49.33h,122.97t/data=!3m7!1e1!3m5!1sHUfp7FBiZu2vK7_NmX_kOw!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-32.97172971729728%26panoid%3DHUfp7FBiZu2vK7_NmX_kOw%26yaw%3D49.33416910035293!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>RUA CONEGO CASSIANO 205, 205, CENTRO</t>
+        </is>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (5.5m, 79 graus) e rumo (31.3m, 63 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G311" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>222494871</t>
+        </is>
+      </c>
+      <c r="B312" t="n">
+        <v>1152</v>
+      </c>
+      <c r="C312" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5906612,-46.9371509,3a,90y,318.26h,120.07t/data=!3m7!1e1!3m5!1sWRj5OW8IxwKAItQJByQwdQ!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-30.065578494925035%26panoid%3DWRj5OW8IxwKAItQJByQwdQ%26yaw%3D318.25788052211084!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>RUA ASTOLFO RODRIGUES 39, 39, CENTRO</t>
+        </is>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (8.0m, 48 graus) e rumo (49.1m, 44 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G312" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>221704112</t>
+        </is>
+      </c>
+      <c r="B313" t="n">
+        <v>1156</v>
+      </c>
+      <c r="C313" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5913529,-46.9371969,3a,90y,159.62h,134.73t/data=!3m7!1e1!3m5!1sTtegEs1bVkrUYTjHNE1_Vw!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-44.73455854163052%26panoid%3DTtegEs1bVkrUYTjHNE1_Vw%26yaw%3D159.62290850230644!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>RUA DOUTOR FRANKLIN DE CASTRO 226, 226, CENTRO</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>confirmar - poste mais proximo (3.9m) tem 72 graus de diferenca de rumo, mas esta perto o suficiente pra ser so ruido de GPS</t>
+        </is>
+      </c>
+      <c r="G313" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>222494875</t>
+        </is>
+      </c>
+      <c r="B314" t="n">
+        <v>1159</v>
+      </c>
+      <c r="C314" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5904643,-46.9381892,3a,90y,297.15h,110.08t/data=!3m7!1e1!3m5!1sw-q1INU0XOaaStCUpSEe2A!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-20.078382395479338%26panoid%3Dw-q1INU0XOaaStCUpSEe2A%26yaw%3D297.15164845151526!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>RUA DOUTOR FRANKLIN DE CASTRO 52, 52, CENTRO</t>
+        </is>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (4.7m, 106 graus) e rumo (40.5m, 65 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G314" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>219993000</t>
+        </is>
+      </c>
+      <c r="B315" t="n">
+        <v>1163</v>
+      </c>
+      <c r="C315" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5909168,-46.9386671,3a,90y,13.59h,131.71t/data=!3m7!1e1!3m5!1sKbyDPXGh_Cm7NTH5ivy0ng!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-41.709841287143774%26panoid%3DKbyDPXGh_Cm7NTH5ivy0ng%26yaw%3D13.589650604395302!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>RUA CALIMERIO GUIMARAES 72, 72, CENTRO</t>
+        </is>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (8.8m, 50 graus) e rumo (67.1m, 34 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G315" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>221704185</t>
+        </is>
+      </c>
+      <c r="B316" t="n">
+        <v>1165</v>
+      </c>
+      <c r="C316" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.591275,-46.9382343,3a,90y,33.98h,137.2t/data=!3m7!1e1!3m5!1sZQQsl4HH5_D5rEYpzkCJSg!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-47.198953002853045%26panoid%3DZQQsl4HH5_D5rEYpzkCJSg%26yaw%3D33.97640668904097!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>RUA CALIMERIO GUIMARAES 120, 120, CENTRO</t>
+        </is>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>confirmar - poste mais proximo (8.0m) tem 73 graus de diferenca de rumo, mas esta perto o suficiente pra ser so ruido de GPS</t>
+        </is>
+      </c>
+      <c r="G316" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>221704223</t>
+        </is>
+      </c>
+      <c r="B317" t="n">
+        <v>1168</v>
+      </c>
+      <c r="C317" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5914732,-46.9397741,3a,75y,165.26h,129.76t/data=!3m7!1e1!3m5!1sBg5-AVShTj3Jd0WI0gOJ6Q!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-39.76044798599278%26panoid%3DBg5-AVShTj3Jd0WI0gOJ6Q%26yaw%3D165.25656284648034!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>RUA DOM JOSE GASPAR 62, 62, CENTRO</t>
+        </is>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>cod_id escolhido pelo rumo, nao pela distancia (mais proximo a 10.9m tinha 96 graus de diferenca de rumo); ATENCAO nome de rua muito diferente: Street View diz o endereco e '428 Av. Antônio Carlos', cod_id escolhido e de 'RUA DOM JOSE GASPAR 62, 62, CENTRO' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G317" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>224223469</t>
+        </is>
+      </c>
+      <c r="B318" t="n">
+        <v>1177</v>
+      </c>
+      <c r="C318" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5922555,-46.9404107,3a,51.5y,34.57h,112.96t/data=!3m7!1e1!3m5!1sy-PMcjEhDBhVnIFEzOK3gQ!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-22.962904410858286%26panoid%3Dy-PMcjEhDBhVnIFEzOK3gQ%26yaw%3D34.573052007741026!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>AVENIDA ANTONIO CARLOS 275, 275, CENTRO</t>
+        </is>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>ATENCAO nome de rua muito diferente: Street View diz o endereco e 'MG-428', cod_id escolhido e de 'AVENIDA ANTONIO CARLOS 275, 275, CENTRO' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G318" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>224495795</t>
+        </is>
+      </c>
+      <c r="B319" t="n">
+        <v>1178</v>
+      </c>
+      <c r="C319" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5923987,-46.94025,3a,48.9y,85.51h,110.74t/data=!3m7!1e1!3m5!1sDoqJK4rzjll8-NTQQ8at4Q!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-20.735015003941953%26panoid%3DDoqJK4rzjll8-NTQQ8at4Q%26yaw%3D85.5126846590248!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D319" t="inlineStr">
+        <is>
+          <t>RUA CAPITAO IZIDRO 0, 0, CENTRO</t>
+        </is>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (15.2m, 29 graus) e rumo (70.6m, 28 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G319" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>222494845</t>
+        </is>
+      </c>
+      <c r="B320" t="n">
+        <v>1180</v>
+      </c>
+      <c r="C320" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5929061,-46.9395438,3a,75y,317.4h,123.78t/data=!3m7!1e1!3m5!1sN9DqVgXy4dGNVZfVnoqh6A!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-33.78023626426142%26panoid%3DN9DqVgXy4dGNVZfVnoqh6A%26yaw%3D317.4000383828405!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D320" t="inlineStr">
+        <is>
+          <t>RUA CAPITAO IZIDRO 97, 97, CENTRO</t>
+        </is>
+      </c>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (11.6m, 14 graus) e rumo (51.3m, 8 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G320" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>223455594</t>
+        </is>
+      </c>
+      <c r="B321" t="n">
+        <v>1181</v>
+      </c>
+      <c r="C321" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5930296,-46.9393993,3a,90y,97.97h,125.26t/data=!3m7!1e1!3m5!1smArsKA7UfOyaCoDH3xruTw!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-35.26355365115391%26panoid%3DmArsKA7UfOyaCoDH3xruTw%26yaw%3D97.96695470173997!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D321" t="inlineStr">
+        <is>
+          <t>RUA CAPITAO IZIDRO 170, 170, CENTRO</t>
+        </is>
+      </c>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (4.3m, 41 graus) e rumo (68.2m, 33 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G321" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>219384994</t>
+        </is>
+      </c>
+      <c r="B322" t="n">
+        <v>1182</v>
+      </c>
+      <c r="C322" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.593275,-46.9390977,3a,90y,38.24h,142.18t/data=!3m7!1e1!3m5!1sCJ6N3xmbufEybYwDa5QatQ!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-52.17723648504733%26panoid%3DCJ6N3xmbufEybYwDa5QatQ%26yaw%3D38.238004137517514!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D322" t="inlineStr">
+        <is>
+          <t>RUA CAPITAO IZIDRO 204, 204, CENTRO</t>
+        </is>
+      </c>
+      <c r="E322" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (1.4m, 145 graus) e rumo (43.7m, 85 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G322" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>224357820</t>
+        </is>
+      </c>
+      <c r="B323" t="n">
+        <v>1184</v>
+      </c>
+      <c r="C323" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5937977,-46.9384645,3a,90y,335.79h,120.51t/data=!3m7!1e1!3m5!1sNmh2K4VJxrUeNQodIBYEcw!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-30.506864993681006%26panoid%3DNmh2K4VJxrUeNQodIBYEcw%26yaw%3D335.794655876032!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D323" t="inlineStr">
+        <is>
+          <t>RUA CAPITAO IZIDRO 280, 280, CENTRO</t>
+        </is>
+      </c>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (10.3m, 38 graus) e rumo (45.3m, 17 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G323" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>904333620</t>
+        </is>
+      </c>
+      <c r="B324" t="n">
+        <v>1185</v>
+      </c>
+      <c r="C324" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5939844,-46.9382425,3a,90y,37.26h,135t/data=!3m7!1e1!3m5!1sNqzgpTTX0LLiRwomQ51Ecw!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-45.00367332452811%26panoid%3DNqzgpTTX0LLiRwomQ51Ecw%26yaw%3D37.263285471847354!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D324" t="inlineStr">
+        <is>
+          <t>RUA CAPITAO IZIDRO 306, 306, CENTRO</t>
+        </is>
+      </c>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>confirmar - poste mais proximo (1.9m) tem 155 graus de diferenca de rumo, mas esta perto o suficiente pra ser so ruido de GPS</t>
+        </is>
+      </c>
+      <c r="G324" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>219387235</t>
+        </is>
+      </c>
+      <c r="B325" t="n">
+        <v>1192</v>
+      </c>
+      <c r="C325" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5943637,-46.9369928,3a,90y,18.59h,127.04t/data=!3m7!1e1!3m5!1s4os9xjhk4HTsi_HrNIdzcA!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-37.04419990971009%26panoid%3D4os9xjhk4HTsi_HrNIdzcA%26yaw%3D18.59355125360136!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D325" t="inlineStr">
+        <is>
+          <t>RUA DOM JOSE GASPAR 420, 420, CENTRO</t>
+        </is>
+      </c>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (4.3m, 50 graus) e rumo (45.8m, 35 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G325" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>223978046</t>
+        </is>
+      </c>
+      <c r="B326" t="n">
+        <v>1203</v>
+      </c>
+      <c r="C326" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5940785,-46.9364049,3a,75y,160.69h,110.44t/data=!3m7!1e1!3m5!1sTMZy_9lUxMJbOLkH7DTVUg!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-20.44364490769263%26panoid%3DTMZy_9lUxMJbOLkH7DTVUg%26yaw%3D160.689835957023!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D326" t="inlineStr">
+        <is>
+          <t>RUA PRESIDENTE OLEGARIO MACIEL 458, 458, CENTRO</t>
+        </is>
+      </c>
+      <c r="E326" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (10.8m, 12 graus) e rumo (45.3m, 11 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G326" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>220854040</t>
+        </is>
+      </c>
+      <c r="B327" t="n">
+        <v>1207</v>
+      </c>
+      <c r="C327" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5931566,-46.9362766,3a,75y,266.59h,119.22t/data=!3m7!1e1!3m5!1saqAUmqmlbO8rCn3Q3HtcGQ!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-29.220566208222664%26panoid%3DaqAUmqmlbO8rCn3Q3HtcGQ%26yaw%3D266.591627330336!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D327" t="inlineStr">
+        <is>
+          <t>RUA ALMEIDA CAMPOS 84, 84, CENTRO</t>
+        </is>
+      </c>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>confirmar - poste mais proximo (8.2m) tem 95 graus de diferenca de rumo, mas esta perto o suficiente pra ser so ruido de GPS</t>
+        </is>
+      </c>
+      <c r="G327" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>219384939</t>
+        </is>
+      </c>
+      <c r="B328" t="n">
+        <v>1211</v>
+      </c>
+      <c r="C328" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5926725,-46.9365962,3a,75y,92.27h,128.72t/data=!3m7!1e1!3m5!1s8VHDBsogE0gvGpXAqosYxA!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-38.71613383240776%26panoid%3D8VHDBsogE0gvGpXAqosYxA%26yaw%3D92.26908988110935!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>RUA CALIMERIO GUIMARAES 360, 360, CENTRO</t>
+        </is>
+      </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (6.7m, 37 graus) e rumo (61.2m, 33 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G328" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>224357700</t>
+        </is>
+      </c>
+      <c r="B329" t="n">
+        <v>1212</v>
+      </c>
+      <c r="C329" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5924807,-46.9368129,3a,90y,16.36h,137.85t/data=!3m7!1e1!3m5!1sT9VTJYafN6BePbVSkC-7LQ!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-47.84671463125744%26panoid%3DT9VTJYafN6BePbVSkC-7LQ%26yaw%3D16.357779893078714!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>RUA CALIMERIO GUIMARAES 326, 326, CENTRO</t>
+        </is>
+      </c>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>confirmar - poste mais proximo (2.0m) tem 78 graus de diferenca de rumo, mas esta perto o suficiente pra ser so ruido de GPS</t>
+        </is>
+      </c>
+      <c r="G329" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>219384952</t>
+        </is>
+      </c>
+      <c r="B330" t="n">
+        <v>1213</v>
+      </c>
+      <c r="C330" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5922298,-46.9371033,3a,90y,34.58h,132.39t/data=!3m7!1e1!3m5!1sOKMUewa_4AdeGF47fldIxA!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-42.38780175591691%26panoid%3DOKMUewa_4AdeGF47fldIxA%26yaw%3D34.57883366767379!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D330" t="inlineStr">
+        <is>
+          <t>RUA CALIMERIO GUIMARAES 302, 302, CENTRO</t>
+        </is>
+      </c>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (1.5m, 146 graus) e rumo (48.1m, 41 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G330" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>220854062</t>
+        </is>
+      </c>
+      <c r="B331" t="n">
+        <v>1221</v>
+      </c>
+      <c r="C331" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5922807,-46.9361515,3a,48.9y,130.59h,118.51t/data=!3m7!1e1!3m5!1szSCPGfR_PEO2SJsxj4qmUQ!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-28.507007996672527%26panoid%3DzSCPGfR_PEO2SJsxj4qmUQ%26yaw%3D130.58793653409862!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>RUA DOUTOR FRANKLIN DE CASTRO 346, 346, CENTRO</t>
+        </is>
+      </c>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (13.5m, 23 graus) e rumo (46.8m, 7 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G331" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>223455913</t>
+        </is>
+      </c>
+      <c r="B332" t="n">
+        <v>1231</v>
+      </c>
+      <c r="C332" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5943922,-46.9344967,3a,90y,13.27h,133.37t/data=!3m7!1e1!3m5!1s5bNh3i2l0fx-NttL3q-obQ!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-43.37459908626559%26panoid%3D5bNh3i2l0fx-NttL3q-obQ%26yaw%3D13.266705642697389!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D332" t="inlineStr">
+        <is>
+          <t>RUA CALIMERIO GUIMARAES 619, 619, CENTRO</t>
+        </is>
+      </c>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (3.3m, 89 graus) e rumo (34.2m, 52 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G332" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>219992931</t>
+        </is>
+      </c>
+      <c r="B333" t="n">
+        <v>1239</v>
+      </c>
+      <c r="C333" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5919556,-46.9355075,3a,90y,67.47h,117.92t/data=!3m7!1e1!3m5!1sw_hdvajDy-ZEg02-nZC4_Q!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-27.9245760719096%26panoid%3Dw_hdvajDy-ZEg02-nZC4_Q%26yaw%3D67.47193809972651!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D333" t="inlineStr">
+        <is>
+          <t>RUA CONEGO CASSIANO 430, 430, CENTRO</t>
+        </is>
+      </c>
+      <c r="E333" t="inlineStr">
+        <is>
+          <t>confirmar - poste mais proximo (2.8m) tem 115 graus de diferenca de rumo, mas esta perto o suficiente pra ser so ruido de GPS</t>
+        </is>
+      </c>
+      <c r="G333" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>219384975</t>
+        </is>
+      </c>
+      <c r="B334" t="n">
+        <v>1245</v>
+      </c>
+      <c r="C334" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5917119,-46.9365279,3a,90y,66.07h,122.83t/data=!3m7!1e1!3m5!1ssWl9BRV5SKGha-W213YsfA!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-32.83341319333691%26panoid%3DsWl9BRV5SKGha-W213YsfA%26yaw%3D66.06527266827302!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D334" t="inlineStr">
+        <is>
+          <t>RUA LIMIRIO AFONSO 21, 21, CENTRO</t>
+        </is>
+      </c>
+      <c r="E334" t="inlineStr">
+        <is>
+          <t>confirmar - poste mais proximo (1.6m) tem 104 graus de diferenca de rumo, mas esta perto o suficiente pra ser so ruido de GPS</t>
+        </is>
+      </c>
+      <c r="G334" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>223455537</t>
+        </is>
+      </c>
+      <c r="B335" t="n">
+        <v>1266</v>
+      </c>
+      <c r="C335" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5949636,-46.9370769,3a,90y,36.33h,126.57t/data=!3m7!1e1!3m5!1sNZCW8qM7BSLKQ27K5JrkXA!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-36.568167294165164%26panoid%3DNZCW8qM7BSLKQ27K5JrkXA%26yaw%3D36.33121675102123!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t>RUA CAPITAO IZIDRO 460, 460, CENTRO</t>
+        </is>
+      </c>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>confirmar - poste mais proximo (2.5m) tem 99 graus de diferenca de rumo, mas esta perto o suficiente pra ser so ruido de GPS</t>
+        </is>
+      </c>
+      <c r="G335" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>223977745</t>
+        </is>
+      </c>
+      <c r="B336" t="n">
+        <v>1272</v>
+      </c>
+      <c r="C336" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5956911,-46.9373612,3a,90y,183.62h,114.29t/data=!3m7!1e1!3m5!1shbIifRyE_ZlP3cHOZZonOw!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-24.289946692254418%26panoid%3DhbIifRyE_ZlP3cHOZZonOw%26yaw%3D183.62233346174662!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t>RUA NOSSA SENHORA DA CONCEICAO 0, 0, CENTRO</t>
+        </is>
+      </c>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (10.9m, 20 graus) e rumo (61.3m, 2 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G336" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>220780224</t>
+        </is>
+      </c>
+      <c r="B337" t="n">
+        <v>1276</v>
+      </c>
+      <c r="C337" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5845449,-46.9397167,3a,90y,353.7h,128.9t/data=!3m7!1e1!3m5!1s4FIrdQVPH8_ytRe7tLwyYA!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-38.89802089381175%26panoid%3D4FIrdQVPH8_ytRe7tLwyYA%26yaw%3D353.70214834042207!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>RUA GERALCINO RIBEIRO DA SILVA 101, 101, SAO PEDRO</t>
+        </is>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (6.4m, 66 graus) e rumo (60.8m, 49 graus) nao concordam com confianca; ATENCAO nome de rua muito diferente: Street View diz o endereco e '418 R. Teófilo dos Santos', cod_id escolhido e de 'RUA GERALCINO RIBEIRO DA SILVA 101, 101, SAO PEDRO' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G337" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>224251161</t>
+        </is>
+      </c>
+      <c r="B338" t="n">
+        <v>1277</v>
+      </c>
+      <c r="C338" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5846787,-46.939527,3a,48.9y,105.98h,119.62t/data=!3m7!1e1!3m5!1s89zNC7lETLq1ZYKKb9pt7Q!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-29.619792920486844%26panoid%3D89zNC7lETLq1ZYKKb9pt7Q%26yaw%3D105.97668527483472!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>RUA TEOFILO DOS SANTOS 373, 373, SAO PEDRO</t>
+        </is>
+      </c>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>confirmar - poste mais proximo (2.6m) tem 79 graus de diferenca de rumo, mas esta perto o suficiente pra ser so ruido de GPS</t>
+        </is>
+      </c>
+      <c r="G338" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>222494803</t>
+        </is>
+      </c>
+      <c r="B339" t="n">
+        <v>1279</v>
+      </c>
+      <c r="C339" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5849405,-46.938999,3a,80.1y,169.75h,123.8t/data=!3m7!1e1!3m5!1sP523mmhYzopo6vFt5jl1TQ!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-33.800910555194264%26panoid%3DP523mmhYzopo6vFt5jl1TQ%26yaw%3D169.74557993953565!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>RUA TEOFILO DOS SANTOS 337, 337, SAO PEDRO</t>
+        </is>
+      </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>ATENCAO nome de rua muito diferente: Street View diz o endereco e '192 R. João Verçosa', cod_id escolhido e de 'RUA TEOFILO DOS SANTOS 337, 337, SAO PEDRO' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente); ATENCAO: numero de poste 'Poste 196' preenchido na planilha nao foi encontrado na base -- usei o match por distancia/rumo/rua como recurso, confirmar</t>
+        </is>
+      </c>
+      <c r="G339" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>219384989</t>
+        </is>
+      </c>
+      <c r="B340" t="n">
+        <v>1280</v>
+      </c>
+      <c r="C340" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5850726,-46.9389728,3a,90y,351.92h,117.39t/data=!3m7!1e1!3m5!1soF4zb2QmZvCi9d6Wge-Gug!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-27.394075253792465%26panoid%3DoF4zb2QmZvCi9d6Wge-Gug%26yaw%3D351.92115678618165!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D340" t="inlineStr">
+        <is>
+          <t>RUA JOAO VERCOSA 178, 178, SAO PEDRO</t>
+        </is>
+      </c>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t>confirmar - poste mais proximo (4.1m) tem 61 graus de diferenca de rumo, mas esta perto o suficiente pra ser so ruido de GPS; ATENCAO nome de rua muito diferente: Street View diz o endereco e '330 R. Teófilo dos Santos', cod_id escolhido e de 'RUA JOAO VERCOSA 178, 178, SAO PEDRO' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente); ATENCAO: numero de poste 'Poste 213' preenchido na planilha nao foi encontrado na base -- usei o match por distancia/rumo/rua como recurso, confirmar</t>
+        </is>
+      </c>
+      <c r="G340" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>223455650</t>
+        </is>
+      </c>
+      <c r="B341" t="n">
+        <v>1281</v>
+      </c>
+      <c r="C341" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5852473,-46.9387349,3a,90y,12.92h,139.94t/data=!3m7!1e1!3m5!1siPXDj8e-gQEuUXS2m-zJcQ!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-49.94329561086303%26panoid%3DiPXDj8e-gQEuUXS2m-zJcQ%26yaw%3D12.922262391139647!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D341" t="inlineStr">
+        <is>
+          <t>RUA TEOFILO DOS SANTOS 285, 285, SAO PEDRO</t>
+        </is>
+      </c>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (7.5m, 66 graus) e rumo (42.9m, 61 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G341" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>223455576</t>
+        </is>
+      </c>
+      <c r="B342" t="n">
+        <v>1286</v>
+      </c>
+      <c r="C342" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5859854,-46.9376713,3a,75y,319.76h,113.84t/data=!3m7!1e1!3m5!1sdYD6hPdUdmR0qIEGw47fBw!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-23.83624330308136%26panoid%3DdYD6hPdUdmR0qIEGw47fBw%26yaw%3D319.76138326808433!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>RUA TEOFILO DOS SANTOS 178, 178, RICA</t>
+        </is>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (12.1m, 20 graus) e rumo (46.5m, 15 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G342" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>222733901</t>
+        </is>
+      </c>
+      <c r="B343" t="n">
+        <v>1287</v>
+      </c>
+      <c r="C343" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5861037,-46.9374992,3a,90y,57.67h,133.24t/data=!3m7!1e1!3m5!1sscGId-q3As4l5Rg8Et8FqA!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-43.235603909521444%26panoid%3DscGId-q3As4l5Rg8Et8FqA%26yaw%3D57.66900756268609!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D343" t="inlineStr">
+        <is>
+          <t>RUA TIA NICA 193, 193, RICA</t>
+        </is>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>confirmar - poste mais proximo (1.7m) tem 78 graus de diferenca de rumo, mas esta perto o suficiente pra ser so ruido de GPS; ATENCAO nome de rua muito diferente: Street View diz o endereco e '142 R. Teófilo dos Santos', cod_id escolhido e de 'RUA TIA NICA 193, 193, RICA' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G343" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>224357723</t>
+        </is>
+      </c>
+      <c r="B344" t="n">
+        <v>1289</v>
+      </c>
+      <c r="C344" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5863401,-46.9371695,3a,75y,95.92h,118.95t/data=!3m7!1e1!3m5!1su4JVB59aj1_-MV9Yi8Swiw!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-28.950015797226953%26panoid%3Du4JVB59aj1_-MV9Yi8Swiw%26yaw%3D95.92127901913652!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D344" t="inlineStr">
+        <is>
+          <t>RUA TEOFILO DOS SANTOS 96, 96, RICA</t>
+        </is>
+      </c>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (0.6m, 47 graus) e rumo (46.4m, 31 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G344" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>219992922</t>
+        </is>
+      </c>
+      <c r="B345" t="n">
+        <v>1290</v>
+      </c>
+      <c r="C345" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5866693,-46.9366939,3a,48.9y,317.56h,105.23t/data=!3m7!1e1!3m5!1s9N7xTwOnhdGIAwNFITxk7w!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-15.234000980907126%26panoid%3D9N7xTwOnhdGIAwNFITxk7w%26yaw%3D317.55565287081015!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t>RUA TEOFILO DOS SANTOS 41, 41, RICA</t>
+        </is>
+      </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (15.5m, 14 graus) e rumo (61.3m, 11 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G345" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>221704093</t>
+        </is>
+      </c>
+      <c r="B346" t="n">
+        <v>1291</v>
+      </c>
+      <c r="C346" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5867968,-46.9365203,3a,77.1y,91.49h,119.49t/data=!3m7!1e1!3m5!1sE6eMZuH4avVhtm2L0hfBHA!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-29.490831004421963%26panoid%3DE6eMZuH4avVhtm2L0hfBHA%26yaw%3D91.48965886532628!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D346" t="inlineStr">
+        <is>
+          <t>RUA PADRE ANCHIETA 387, 387, RICA</t>
+        </is>
+      </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (5.2m, 44 graus) e rumo (38.8m, 37 graus) nao concordam com confianca; ATENCAO nome de rua muito diferente: Street View diz o endereco e '27 R. Teófilo dos Santos', cod_id escolhido e de 'RUA PADRE ANCHIETA 387, 387, RICA' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G346" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>222494764</t>
+        </is>
+      </c>
+      <c r="B347" t="n">
+        <v>1292</v>
+      </c>
+      <c r="C347" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5870354,-46.9361821,3a,90y,34.42h,138.32t/data=!3m7!1e1!3m5!1sEVF-ySLUQb9Nbr9lD52Y5Q!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-48.32479404868988%26panoid%3DEVF-ySLUQb9Nbr9lD52Y5Q%26yaw%3D34.41794523794839!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D347" t="inlineStr">
+        <is>
+          <t>RUA ITACURU 216, 216, CENTRO</t>
+        </is>
+      </c>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (5.6m, 99 graus) e rumo (51.8m, 46 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G347" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>222495131</t>
+        </is>
+      </c>
+      <c r="B348" t="n">
+        <v>1294</v>
+      </c>
+      <c r="C348" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5875115,-46.9355856,3a,75y,332.77h,117.26t/data=!3m7!1e1!3m5!1sg-lw956zeoSEaChMW1pyIA!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-27.25754693365475%26panoid%3Dg-lw956zeoSEaChMW1pyIA%26yaw%3D332.77207419290085!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D348" t="inlineStr">
+        <is>
+          <t>RUA ITACURU 145, 145, CENTRO</t>
+        </is>
+      </c>
+      <c r="E348" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (12.7m, 26 graus) e rumo (53.9m, 24 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G348" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>221704417</t>
+        </is>
+      </c>
+      <c r="B349" t="n">
+        <v>1296</v>
+      </c>
+      <c r="C349" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5880337,-46.9350863,3a,48.9y,333.06h,110.47t/data=!3m7!1e1!3m5!1sRPoSyl6Byhgc1vsNTPJBBw!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-20.4722399368421%26panoid%3DRPoSyl6Byhgc1vsNTPJBBw%26yaw%3D333.05711521249486!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D349" t="inlineStr">
+        <is>
+          <t>RUA ITACURU 73, 73, CENTRO</t>
+        </is>
+      </c>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (14.8m, 17 graus) e rumo (38.9m, 15 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G349" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>224357743</t>
+        </is>
+      </c>
+      <c r="B350" t="n">
+        <v>1301</v>
+      </c>
+      <c r="C350" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.587233,-46.9369265,3a,52y,103.4h,104.4t/data=!3m8!1e1!3m6!1sQGgsgR-FdOWf7kcZb3m5Pw!2e0!5s20110701T000000!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-14.398789541719125%26panoid%3DQGgsgR-FdOWf7kcZb3m5Pw%26yaw%3D103.40036288434973!7i13312!8i6656?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D350" t="inlineStr">
+        <is>
+          <t>RUA PADRE ANCHIETA 323, 323, RICA</t>
+        </is>
+      </c>
+      <c r="E350" t="inlineStr">
+        <is>
+          <t>ATENCAO nome de rua muito diferente: Street View diz o endereco e '20 R. Abdanur Elías', cod_id escolhido e de 'RUA PADRE ANCHIETA 323, 323, RICA' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G350" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>219384926</t>
+        </is>
+      </c>
+      <c r="B351" t="n">
+        <v>1317</v>
+      </c>
+      <c r="C351" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5888959,-46.9380275,3a,90y,243.55h,120.1t/data=!3m7!1e1!3m5!1sp0-P8gkyxJOYlPivb19RJQ!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-30.104699711091186%26panoid%3Dp0-P8gkyxJOYlPivb19RJQ%26yaw%3D243.55471694249104!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>RUA PADRE ANCHIETA 0, 0, CENTRO</t>
+        </is>
+      </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>ATENCAO nome de rua muito diferente: Street View diz o endereco e '95 Av. Antônio Carlos', cod_id escolhido e de 'RUA PADRE ANCHIETA 0, 0, CENTRO' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G351" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>223455638</t>
+        </is>
+      </c>
+      <c r="B352" t="n">
+        <v>1318</v>
+      </c>
+      <c r="C352" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5886978,-46.9380196,3a,90y,89.48h,121.7t/data=!3m7!1e1!3m5!1sGTLour3Pcr52dw86nb7jqQ!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-31.696103098558012%26panoid%3DGTLour3Pcr52dw86nb7jqQ%26yaw%3D89.48445825419495!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr">
+        <is>
+          <t>RUA MARIO CAMPOS 6, 6, CENTRO</t>
+        </is>
+      </c>
+      <c r="E352" t="inlineStr">
+        <is>
+          <t>confirmar - poste mais proximo (2.0m) tem 136 graus de diferenca de rumo, mas esta perto o suficiente pra ser so ruido de GPS</t>
+        </is>
+      </c>
+      <c r="G352" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>222494827</t>
+        </is>
+      </c>
+      <c r="B353" t="n">
+        <v>1319</v>
+      </c>
+      <c r="C353" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5885334,-46.9382783,3a,90y,82.4h,133.75t/data=!3m7!1e1!3m5!1sKt6ZN0xc3aGLvTo23jrllw!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-43.750211856629164%26panoid%3DKt6ZN0xc3aGLvTo23jrllw%26yaw%3D82.40223866281475!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t>RUA MARIO CAMPOS 40, 40, CENTRO</t>
+        </is>
+      </c>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t>confirmar - poste mais proximo (2.1m) tem 180 graus de diferenca de rumo, mas esta perto o suficiente pra ser so ruido de GPS</t>
+        </is>
+      </c>
+      <c r="G353" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>221704213</t>
+        </is>
+      </c>
+      <c r="B354" t="n">
+        <v>1320</v>
+      </c>
+      <c r="C354" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5884327,-46.938439,3a,49.6y,313.17h,109.43t/data=!3m7!1e1!3m5!1snDDxoh_fj8wG4QLZlMB4cA!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-19.434163483438255%26panoid%3DnDDxoh_fj8wG4QLZlMB4cA%26yaw%3D313.1707412768292!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D354" t="inlineStr">
+        <is>
+          <t>RUA MARIO CAMPOS 93, 93, CENTRO</t>
+        </is>
+      </c>
+      <c r="E354" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (13.8m, 13 graus) e rumo (46.6m, 12 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G354" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>219385048</t>
+        </is>
+      </c>
+      <c r="B355" t="n">
+        <v>1325</v>
+      </c>
+      <c r="C355" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5877829,-46.9393558,3a,90y,112.36h,132.69t/data=!3m7!1e1!3m5!1sQKmx5Yc_n8GyPM09D4bqGg!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-42.68772027843633%26panoid%3DQKmx5Yc_n8GyPM09D4bqGg%26yaw%3D112.3603407754911!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D355" t="inlineStr">
+        <is>
+          <t>RUA MARIO CAMPOS 186, 186, CENTRO</t>
+        </is>
+      </c>
+      <c r="E355" t="inlineStr">
+        <is>
+          <t>confirmar - poste mais proximo (3.0m) tem 113 graus de diferenca de rumo, mas esta perto o suficiente pra ser so ruido de GPS; ATENCAO nome de rua muito diferente: Street View diz o endereco e '119 R. Manoel Francisco', cod_id escolhido e de 'RUA MARIO CAMPOS 186, 186, CENTRO' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G355" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>224357798</t>
+        </is>
+      </c>
+      <c r="B356" t="n">
+        <v>1333</v>
+      </c>
+      <c r="C356" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5859608,-46.9386868,3a,90y,138.97h,113.79t/data=!3m7!1e1!3m5!1smkGB5_A96M5pgwGkG-FuJw!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-23.786228351767335%26panoid%3DmkGB5_A96M5pgwGkG-FuJw%26yaw%3D138.96640815645864!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D356" t="inlineStr">
+        <is>
+          <t>PRACA MARIA BITTAR DE REZENDE 200, 200, SAO PEDRO</t>
+        </is>
+      </c>
+      <c r="E356" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (5.7m, 52 graus) e rumo (12.8m, 33 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G356" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>224357800</t>
+        </is>
+      </c>
+      <c r="B357" t="n">
+        <v>1335</v>
+      </c>
+      <c r="C357" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5857181,-46.9384862,3a,90y,145.66h,132.71t/data=!3m7!1e1!3m5!1sjX8w8ZUKSJ-N6S6UMfFG0A!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-42.7142788283995%26panoid%3DjX8w8ZUKSJ-N6S6UMfFG0A%26yaw%3D145.66497130882223!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D357" t="inlineStr">
+        <is>
+          <t>PRACA MARIA BITTAR DE REZENDE 200, 200, SAO PEDRO</t>
+        </is>
+      </c>
+      <c r="E357" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (5.5m, 65 graus) e rumo (44.1m, 60 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G357" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>224318216</t>
+        </is>
+      </c>
+      <c r="B358" t="n">
+        <v>1338</v>
+      </c>
+      <c r="C358" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5852201,-46.9391336,3a,75y,171.3h,117.53t/data=!3m7!1e1!3m5!1spMQx7vQy9Cv5qaQe52Ri0A!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-27.53137954822516%26panoid%3DpMQx7vQy9Cv5qaQe52Ri0A%26yaw%3D171.30266444002305!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D358" t="inlineStr">
+        <is>
+          <t>RUA JOAO VERCOSA 149, 149, SAO PEDRO</t>
+        </is>
+      </c>
+      <c r="E358" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (11.0m, 43 graus) e rumo (44.6m, 35 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G358" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>222494574</t>
+        </is>
+      </c>
+      <c r="B359" t="n">
+        <v>1339</v>
+      </c>
+      <c r="C359" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5854851,-46.9392504,3a,72.1y,173.46h,109.19t/data=!3m7!1e1!3m5!1sR4rvktB4T5O_k3YhBBeegg!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-19.18555693291671%26panoid%3DR4rvktB4T5O_k3YhBBeegg%26yaw%3D173.45546719666507!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D359" t="inlineStr">
+        <is>
+          <t>RUA JOAO VERCOSA 115, 115, SAO PEDRO</t>
+        </is>
+      </c>
+      <c r="E359" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (12.9m, 41 graus) e rumo (51.4m, 32 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G359" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>219991667</t>
+        </is>
+      </c>
+      <c r="B360" t="n">
+        <v>1340</v>
+      </c>
+      <c r="C360" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5858278,-46.9394062,3a,75y,173.33h,109.69t/data=!3m7!1e1!3m5!1slep5qGrSHdFQFKVUNOw-Tg!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-19.68971153151425%26panoid%3Dlep5qGrSHdFQFKVUNOw-Tg%26yaw%3D173.32643467003015!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D360" t="inlineStr">
+        <is>
+          <t>RUA JOAO VERCOSA 267, 267, SAO PEDRO</t>
+        </is>
+      </c>
+      <c r="E360" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (10.0m, 39 graus) e rumo (50.4m, 32 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G360" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>219298231</t>
+        </is>
+      </c>
+      <c r="B361" t="n">
+        <v>1341</v>
+      </c>
+      <c r="C361" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5861585,-46.9396272,3a,75y,136.41h,109.99t/data=!3m7!1e1!3m5!1sMamKuCfSN_KeWIu06Avstw!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-19.991651877614956%26panoid%3DMamKuCfSN_KeWIu06Avstw%26yaw%3D136.41168676709003!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D361" t="inlineStr">
+        <is>
+          <t>RUA JOAO VERCOSA 59, 59, SAO PEDRO</t>
+        </is>
+      </c>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t>ATENCAO nome de rua muito diferente: Street View diz o endereco e '7 R. Américo Autran', cod_id escolhido e de 'RUA JOAO VERCOSA 59, 59, SAO PEDRO' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G361" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>220854135</t>
+        </is>
+      </c>
+      <c r="B362" t="n">
+        <v>1343</v>
+      </c>
+      <c r="C362" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.586827,-46.9393866,3a,90y,68.56h,122.1t/data=!3m7!1e1!3m5!1s-OUzY1KWVYJZvQQI9qH88w!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-32.09964576823772%26panoid%3D-OUzY1KWVYJZvQQI9qH88w%26yaw%3D68.56174475952812!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D362" t="inlineStr">
+        <is>
+          <t>RUA PROFESSOR SATURNINO TEIXEIRA 9, 9, SAO PEDRO</t>
+        </is>
+      </c>
+      <c r="E362" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (3.0m, 125 graus) e rumo (25.6m, 49 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G362" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>350236657</t>
+        </is>
+      </c>
+      <c r="B363" t="n">
+        <v>1349</v>
+      </c>
+      <c r="C363" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5869046,-46.9399212,3a,90y,123.23h,129.72t/data=!3m7!1e1!3m5!1su8RtqWkYDY_jGTXg5lwkQA!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-39.72073208367084%26panoid%3Du8RtqWkYDY_jGTXg5lwkQA%26yaw%3D123.22743698731256!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D363" t="inlineStr">
+        <is>
+          <t>RUA IMBIACA 303, 303, CENTRO</t>
+        </is>
+      </c>
+      <c r="E363" t="inlineStr">
+        <is>
+          <t>confirmar - poste mais proximo (2.5m) tem 61 graus de diferenca de rumo, mas esta perto o suficiente pra ser so ruido de GPS; ATENCAO nome de rua muito diferente: Street View diz o endereco e '145 R. Bom Jardim', cod_id escolhido e de 'RUA IMBIACA 303, 303, CENTRO' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G363" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>350236672</t>
+        </is>
+      </c>
+      <c r="B364" t="n">
+        <v>1353</v>
+      </c>
+      <c r="C364" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5859749,-46.9410328,3a,24.9y,297.18h,102.12t/data=!3m7!1e1!3m5!1suz73NEsupM9H2NvzxzAbVw!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-12.122941522193543%26panoid%3Duz73NEsupM9H2NvzxzAbVw%26yaw%3D297.17640148234364!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D364" t="inlineStr">
+        <is>
+          <t>RUA BENTO ANTONIO 149, 149, CENTRO</t>
+        </is>
+      </c>
+      <c r="E364" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (18.5m, 11 graus) e rumo (26.3m, 7 graus) nao concordam com confianca; ATENCAO nome de rua muito diferente: Street View diz o endereco e '540 R. Imbiaca', cod_id escolhido e de 'RUA BENTO ANTONIO 149, 149, CENTRO' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G364" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>224318325</t>
+        </is>
+      </c>
+      <c r="B365" t="n">
+        <v>1355</v>
+      </c>
+      <c r="C365" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5854677,-46.9415482,3a,48.9y,266.13h,105.92t/data=!3m7!1e1!3m5!1skS2XEJ0vL8QSpqa17vsnYA!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-15.920205344014335%26panoid%3DkS2XEJ0vL8QSpqa17vsnYA%26yaw%3D266.13250446617894!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D365" t="inlineStr">
+        <is>
+          <t>RUA IMBIACA 629, 629, CENTRO</t>
+        </is>
+      </c>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (16.1m, 5 graus) e rumo (50.4m, 2 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G365" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>223977006</t>
+        </is>
+      </c>
+      <c r="B366" t="n">
+        <v>1356</v>
+      </c>
+      <c r="C366" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5854125,-46.9417599,3a,90y,143.94h,129.5t/data=!3m7!1e1!3m5!1sst_bxdw9rU4QfNna18s3VQ!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-39.500181853906724%26panoid%3Dst_bxdw9rU4QfNna18s3VQ%26yaw%3D143.93809611724055!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D366" t="inlineStr">
+        <is>
+          <t>RUA IMBIACA 629, 629, CENTRO</t>
+        </is>
+      </c>
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>confirmar - poste mais proximo (6.7m) tem 83 graus de diferenca de rumo, mas esta perto o suficiente pra ser so ruido de GPS</t>
+        </is>
+      </c>
+      <c r="G366" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>222494608</t>
+        </is>
+      </c>
+      <c r="B367" t="n">
+        <v>1367</v>
+      </c>
+      <c r="C367" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5858052,-46.9431872,3a,90y,9.76h,117.76t/data=!3m7!1e1!3m5!1sR-W1HBlU4jLBFOHtBbSLDw!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-27.7613495783891%26panoid%3DR-W1HBlU4jLBFOHtBbSLDw%26yaw%3D9.7590146633893!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D367" t="inlineStr">
+        <is>
+          <t>RUA MARIO CAMPOS 646, 646, CENTRO</t>
+        </is>
+      </c>
+      <c r="E367" t="inlineStr">
+        <is>
+          <t>confirmar - poste mais proximo (3.9m) tem 76 graus de diferenca de rumo, mas esta perto o suficiente pra ser so ruido de GPS</t>
+        </is>
+      </c>
+      <c r="G367" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>224318280</t>
+        </is>
+      </c>
+      <c r="B368" t="n">
+        <v>1368</v>
+      </c>
+      <c r="C368" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5859231,-46.9429129,3a,75y,88.71h,104.8t/data=!3m7!1e1!3m5!1sJjMgKOn4--XuE9OtKRVTfw!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-14.804884850638345%26panoid%3DJjMgKOn4--XuE9OtKRVTfw%26yaw%3D88.71340825318082!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D368" t="inlineStr">
+        <is>
+          <t>RUA MARIO CAMPOS 612, 612, CENTRO</t>
+        </is>
+      </c>
+      <c r="E368" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (5.9m, 42 graus) e rumo (41.5m, 31 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G368" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>219991729</t>
+        </is>
+      </c>
+      <c r="B369" t="n">
+        <v>1369</v>
+      </c>
+      <c r="C369" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5860388,-46.9426429,3a,48.9y,104.39h,103.89t/data=!3m7!1e1!3m5!1sYb4ZRasa5_d0HQWqiPP6vQ!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-13.893633423754949%26panoid%3DYb4ZRasa5_d0HQWqiPP6vQ%26yaw%3D104.39177155394114!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D369" t="inlineStr">
+        <is>
+          <t>RUA MARIO CAMPOS 557, 557, CENTRO</t>
+        </is>
+      </c>
+      <c r="E369" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (10.8m, 29 graus) e rumo (53.4m, 15 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G369" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>222494606</t>
+        </is>
+      </c>
+      <c r="B370" t="n">
+        <v>1371</v>
+      </c>
+      <c r="C370" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5862372,-46.942203,3a,90y,74.34h,112.51t/data=!3m7!1e1!3m5!1s8t5_VlRkHZhJjok5BaiCIg!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-22.5147167639592%26panoid%3D8t5_VlRkHZhJjok5BaiCIg%26yaw%3D74.34077609284509!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D370" t="inlineStr">
+        <is>
+          <t>RUA MARIO CAMPOS 503, 503, CENTRO</t>
+        </is>
+      </c>
+      <c r="E370" t="inlineStr">
+        <is>
+          <t>confirmar - poste mais proximo (3.9m) tem 97 graus de diferenca de rumo, mas esta perto o suficiente pra ser so ruido de GPS</t>
+        </is>
+      </c>
+      <c r="G370" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>219298312</t>
+        </is>
+      </c>
+      <c r="B371" t="n">
+        <v>1372</v>
+      </c>
+      <c r="C371" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5864073,-46.9418597,3a,75y,61.72h,122.3t/data=!3m7!1e1!3m5!1s9fh7DZ9z7BPe-2CJa6SzHA!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-32.29703980423537%26panoid%3D9fh7DZ9z7BPe-2CJa6SzHA%26yaw%3D61.719800459478016!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D371" t="inlineStr">
+        <is>
+          <t>RUA BENTO ANTONIO 71, 71, CENTRO</t>
+        </is>
+      </c>
+      <c r="E371" t="inlineStr">
+        <is>
+          <t>confirmar - poste mais proximo (2.5m) tem 133 graus de diferenca de rumo, mas esta perto o suficiente pra ser so ruido de GPS; ATENCAO nome de rua muito diferente: Street View diz o endereco e '482 R. Mario Campos', cod_id escolhido e de 'RUA BENTO ANTONIO 71, 71, CENTRO' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G371" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>588535656</t>
+        </is>
+      </c>
+      <c r="B372" t="n">
+        <v>1378</v>
+      </c>
+      <c r="C372" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5868905,-46.9409311,3a,75y,87.01h,114.78t/data=!3m7!1e1!3m5!1sGzyc3CJQtv9Kg9LOev-9VQ!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-24.784712208143347%26panoid%3DGzyc3CJQtv9Kg9LOev-9VQ%26yaw%3D87.0054113695566!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D372" t="inlineStr">
+        <is>
+          <t>RUA MARIO CAMPOS 363, 363, CENTRO</t>
+        </is>
+      </c>
+      <c r="E372" t="inlineStr">
+        <is>
+          <t>confirmar - poste mais proximo (5.6m) tem 69 graus de diferenca de rumo, mas esta perto o suficiente pra ser so ruido de GPS</t>
+        </is>
+      </c>
+      <c r="G372" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>219298313</t>
+        </is>
+      </c>
+      <c r="B373" t="n">
+        <v>1379</v>
+      </c>
+      <c r="C373" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5870355,-46.9406793,3a,48.9y,104.48h,102.48t/data=!3m7!1e1!3m5!1sTwU4Z9kwxAZWPXQih-RLkw!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-12.481988997756801%26panoid%3DTwU4Z9kwxAZWPXQih-RLkw%26yaw%3D104.48185078063703!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D373" t="inlineStr">
+        <is>
+          <t>RUA MARIO CAMPOS 313, 313, CENTRO</t>
+        </is>
+      </c>
+      <c r="E373" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (10.6m, 30 graus) e rumo (36.8m, 20 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G373" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>221704226</t>
+        </is>
+      </c>
+      <c r="B374" t="n">
+        <v>1381</v>
+      </c>
+      <c r="C374" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5873166,-46.9401999,3a,75y,167.57h,109.68t/data=!3m7!1e1!3m5!1sZJjPepwPjMC9noGS8N-wMA!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-19.682846016387032%26panoid%3DZJjPepwPjMC9noGS8N-wMA%26yaw%3D167.57132204199158!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D374" t="inlineStr">
+        <is>
+          <t>RUA BOM JARDIM 95, 95, CENTRO</t>
+        </is>
+      </c>
+      <c r="E374" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (10.2m, 30 graus) e rumo (10.5m, 29 graus) nao concordam com confianca; ATENCAO nome de rua muito diferente: Street View diz o endereco e '269 R. Mario Campos', cod_id escolhido e de 'RUA BOM JARDIM 95, 95, CENTRO' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G374" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>223455619</t>
+        </is>
+      </c>
+      <c r="B375" t="n">
+        <v>1382</v>
+      </c>
+      <c r="C375" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5873724,-46.9401138,3a,90y,7.81h,133.15t/data=!3m7!1e1!3m5!1s-anoTWkSIsSfLChkKrozAw!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-43.148855160952564%26panoid%3D-anoTWkSIsSfLChkKrozAw%26yaw%3D7.808668973411392!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D375" t="inlineStr">
+        <is>
+          <t>RUA BOM JARDIM 98, 98, CENTRO</t>
+        </is>
+      </c>
+      <c r="E375" t="inlineStr">
+        <is>
+          <t>confirmar - poste mais proximo (2.6m) tem 137 graus de diferenca de rumo, mas esta perto o suficiente pra ser so ruido de GPS; ATENCAO nome de rua muito diferente: Street View diz o endereco e '269 R. Mario Campos', cod_id escolhido e de 'RUA BOM JARDIM 98, 98, CENTRO' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G375" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>220854136</t>
+        </is>
+      </c>
+      <c r="B376" t="n">
+        <v>1385</v>
+      </c>
+      <c r="C376" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5875432,-46.9403286,3a,90y,186.94h,113.06t/data=!3m7!1e1!3m5!1s3ipXDFAUxwOpaCHF32hNlg!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-23.05506460193932%26panoid%3D3ipXDFAUxwOpaCHF32hNlg%26yaw%3D186.9435190267189!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>RUA BOM JARDIM 74, 74, CENTRO</t>
+        </is>
+      </c>
+      <c r="E376" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (10.1m, 35 graus) e rumo (41.1m, 29 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G376" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>219992984</t>
+        </is>
+      </c>
+      <c r="B377" t="n">
+        <v>1386</v>
+      </c>
+      <c r="C377" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5877655,-46.9404958,3a,75y,186.73h,102.69t/data=!3m7!1e1!3m5!1stU_KNDJYBBTFPkszpW6nqg!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-12.689850154431838%26panoid%3DtU_KNDJYBBTFPkszpW6nqg%26yaw%3D186.72743323621708!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>RUA BOM JARDIM 46, 46, CENTRO</t>
+        </is>
+      </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (10.8m, 30 graus) e rumo (52.0m, 22 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G377" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>223977847</t>
+        </is>
+      </c>
+      <c r="B378" t="n">
+        <v>1389</v>
+      </c>
+      <c r="C378" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5892573,-46.9392534,3a,48.9y,266.23h,103.8t/data=!3m7!1e1!3m5!1sjAI3Um3rtYQctL4PDb_U9w!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-13.802052297137237%26panoid%3DjAI3Um3rtYQctL4PDb_U9w%26yaw%3D266.2343956063306!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D378" t="inlineStr">
+        <is>
+          <t>AVENIDA VEREADOR JOAO SENA 52, 52, CENTRO</t>
+        </is>
+      </c>
+      <c r="E378" t="inlineStr">
+        <is>
+          <t>confirmar - poste mais proximo (2.3m) tem 175 graus de diferenca de rumo, mas esta perto o suficiente pra ser so ruido de GPS</t>
+        </is>
+      </c>
+      <c r="G378" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>223977849</t>
+        </is>
+      </c>
+      <c r="B379" t="n">
+        <v>1393</v>
+      </c>
+      <c r="C379" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5890063,-46.9397291,3a,90y,250.68h,112.77t/data=!3m7!1e1!3m5!1sgYJ_WkdZoKw0CAKVoRss_A!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-22.771813053775944%26panoid%3DgYJ_WkdZoKw0CAKVoRss_A%26yaw%3D250.67972271460383!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D379" t="inlineStr">
+        <is>
+          <t>AVENIDA VEREADOR JOAO SENA 165, 165, CENTRO</t>
+        </is>
+      </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>ATENCAO nome de rua muito diferente: Street View diz o endereco e '10 R. Maj. Tito', cod_id escolhido e de 'AVENIDA VEREADOR JOAO SENA 165, 165, CENTRO' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G379" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>224318264</t>
+        </is>
+      </c>
+      <c r="B380" t="n">
+        <v>1397</v>
+      </c>
+      <c r="C380" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5883966,-46.9404357,3a,90y,346.22h,107.22t/data=!3m7!1e1!3m5!1swPFbWCnO00Mx8HPZXVQZmA!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-17.221689612804752%26panoid%3DwPFbWCnO00Mx8HPZXVQZmA%26yaw%3D346.21814334659854!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>AVENIDA VEREADOR JOAO SENA 266, 266, CENTRO</t>
+        </is>
+      </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (13.3m, 38 graus) e rumo (46.5m, 32 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G380" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>219385030</t>
+        </is>
+      </c>
+      <c r="B381" t="n">
+        <v>1400</v>
+      </c>
+      <c r="C381" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5880709,-46.9407455,3a,90y,112.94h,131.83t/data=!3m7!1e1!3m5!1sGXq8Qa2Cv78_9fbd_Xv4Mw!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-41.82804509550439%26panoid%3DGXq8Qa2Cv78_9fbd_Xv4Mw%26yaw%3D112.9407193181317!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t>AVENIDA VEREADOR JOAO SENA 296, 296, CENTRO</t>
+        </is>
+      </c>
+      <c r="E381" t="inlineStr">
+        <is>
+          <t>confirmar - poste mais proximo (3.6m) tem 78 graus de diferenca de rumo, mas esta perto o suficiente pra ser so ruido de GPS; ATENCAO nome de rua muito diferente: Street View diz o endereco e '7 R. Bom Jardim', cod_id escolhido e de 'AVENIDA VEREADOR JOAO SENA 296, 296, CENTRO' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G381" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>221621788</t>
+        </is>
+      </c>
+      <c r="B382" t="n">
+        <v>1404</v>
+      </c>
+      <c r="C382" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5874858,-46.941672,3a,75y,65.26h,119.18t/data=!3m7!1e1!3m5!1sQ_ZdqA9kF_OiXI-wfVRcwQ!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-29.184483535187823%26panoid%3DQ_ZdqA9kF_OiXI-wfVRcwQ%26yaw%3D65.25797575942306!7i13312!8i6656?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D382" t="inlineStr">
+        <is>
+          <t>AVENIDA VEREADOR JOAO SENA 460, 460, CENTRO</t>
+        </is>
+      </c>
+      <c r="E382" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (1.9m, 86 graus) e rumo (41.2m, 62 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G382" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>223390302</t>
+        </is>
+      </c>
+      <c r="B383" t="n">
+        <v>1406</v>
+      </c>
+      <c r="C383" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5869749,-46.9420956,3a,75y,238.25h,108.52t/data=!3m7!1e1!3m5!1s7nTJa-yiJYmotTDBR7MNXQ!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-18.52263950618095%26panoid%3D7nTJa-yiJYmotTDBR7MNXQ%26yaw%3D238.25108797696333!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D383" t="inlineStr">
+        <is>
+          <t>AVENIDA VEREADOR JOAO SENA 530, 530, CENTRO</t>
+        </is>
+      </c>
+      <c r="E383" t="inlineStr">
+        <is>
+          <t>ATENCAO nome de rua muito diferente: Street View diz o endereco e '16 R. Bento Antônio', cod_id escolhido e de 'AVENIDA VEREADOR JOAO SENA 530, 530, CENTRO' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G383" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>219991958</t>
+        </is>
+      </c>
+      <c r="B384" t="n">
+        <v>1414</v>
+      </c>
+      <c r="C384" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5858519,-46.9436879,3a,46.3y,291.29h,100.68t/data=!3m7!1e1!3m5!1spe_zyJvgB5yIxXePA_esqw!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-10.684443810832633%26panoid%3Dpe_zyJvgB5yIxXePA_esqw%26yaw%3D291.29420120923294!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D384" t="inlineStr">
+        <is>
+          <t>AVENIDA VEREADOR JOAO SENA 764, 764, CENTRO</t>
+        </is>
+      </c>
+      <c r="E384" t="inlineStr">
+        <is>
+          <t>cod_id escolhido pelo rumo, nao pela distancia (mais proximo a 14.1m tinha 122 graus de diferenca de rumo); ATENCAO nome de rua muito diferente: Street View diz o endereco e '163 R. Ipiao', cod_id escolhido e de 'AVENIDA VEREADOR JOAO SENA 764, 764, CENTRO' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G384" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>219298389</t>
+        </is>
+      </c>
+      <c r="B385" t="n">
+        <v>1422</v>
+      </c>
+      <c r="C385" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5847233,-46.9437195,3a,75y,297.45h,109.12t/data=!3m7!1e1!3m5!1sQ1-UNATpxMeMXx6e2s7SQQ!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-19.118764855378757%26panoid%3DQ1-UNATpxMeMXx6e2s7SQQ%26yaw%3D297.4519930382813!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D385" t="inlineStr">
+        <is>
+          <t>AVENIDA JOAO PAULO II 5, 5, CENTRO</t>
+        </is>
+      </c>
+      <c r="E385" t="inlineStr">
+        <is>
+          <t>ATENCAO nome de rua muito diferente: Street View diz o endereco e '972 R. Ipiao', cod_id escolhido e de 'AVENIDA JOAO PAULO II 5, 5, CENTRO' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G385" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>224318381</t>
+        </is>
+      </c>
+      <c r="B386" t="n">
+        <v>1423</v>
+      </c>
+      <c r="C386" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5844329,-46.9438098,3a,90y,253.35h,108.28t/data=!3m7!1e1!3m5!1sgxojuFsszd4S4ExZ_TfC2g!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-18.277973700406633%26panoid%3DgxojuFsszd4S4ExZ_TfC2g%26yaw%3D253.35310755979953!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D386" t="inlineStr">
+        <is>
+          <t>AVENIDA JOAO PAULO II 5, 5, CENTRO</t>
+        </is>
+      </c>
+      <c r="E386" t="inlineStr">
+        <is>
+          <t>ATENCAO nome de rua muito diferente: Street View diz o endereco e '998 R. Ipiao', cod_id escolhido e de 'AVENIDA JOAO PAULO II 5, 5, CENTRO' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G386" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>221621825</t>
+        </is>
+      </c>
+      <c r="B387" t="n">
+        <v>1428</v>
+      </c>
+      <c r="C387" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5864554,-46.9431402,3a,90y,213.11h,130.63t/data=!3m7!1e1!3m5!1se-P2JKe-h8P7_Yf8s0o25Q!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-40.63495973717724%26panoid%3De-P2JKe-h8P7_Yf8s0o25Q%26yaw%3D213.1054927977276!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D387" t="inlineStr">
+        <is>
+          <t>RUA JOAQUIM ANTONIO DUTRA 30, 30, CENTRO</t>
+        </is>
+      </c>
+      <c r="E387" t="inlineStr">
+        <is>
+          <t>ATENCAO nome de rua muito diferente: Street View diz o endereco e '236 Av. Ver. João Sena', cod_id escolhido e de 'RUA JOAQUIM ANTONIO DUTRA 30, 30, CENTRO' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G387" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>222494674</t>
+        </is>
+      </c>
+      <c r="B388" t="n">
+        <v>1429</v>
+      </c>
+      <c r="C388" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5866196,-46.9429292,3a,90y,166.38h,121.6t/data=!3m7!1e1!3m5!1sb0IenZU0QZT1LF8706ZZmA!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-31.59770036723718%26panoid%3Db0IenZU0QZT1LF8706ZZmA%26yaw%3D166.38115801865473!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D388" t="inlineStr">
+        <is>
+          <t>AVENIDA VEREADOR JOAO SENA 473, 473, CENTRO</t>
+        </is>
+      </c>
+      <c r="E388" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (14.0m, 25 graus) e rumo (38.2m, 20 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G388" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>223976929</t>
+        </is>
+      </c>
+      <c r="B389" t="n">
+        <v>1437</v>
+      </c>
+      <c r="C389" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5878526,-46.9415375,3a,75y,143.83h,115.93t/data=!3m7!1e1!3m5!1sNLVmmTxzE6ZWJhEFWzI6tg!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-25.93148089069419%26panoid%3DNLVmmTxzE6ZWJhEFWzI6tg%26yaw%3D143.83255817446513!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D389" t="inlineStr">
+        <is>
+          <t>RUA DOUTOR BARACUHY 9, 9, CENTRO</t>
+        </is>
+      </c>
+      <c r="E389" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (8.7m, 108 graus) e rumo (8.8m, 38 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G389" t="inlineStr">
         <is>
           <t>BAIXA CONFIANCA - REVISAO</t>
         </is>
@@ -8159,6 +12359,146 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C247" r:id="rId246"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C248" r:id="rId247"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C249" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C250" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C251" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C252" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C253" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C254" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C255" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C256" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C257" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C258" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C259" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C260" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C261" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C262" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C263" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C264" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C265" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C266" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C267" r:id="rId266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C268" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C269" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C270" r:id="rId269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C271" r:id="rId270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C272" r:id="rId271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C273" r:id="rId272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C274" r:id="rId273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C275" r:id="rId274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C276" r:id="rId275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C277" r:id="rId276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C278" r:id="rId277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C279" r:id="rId278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C280" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C281" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C282" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C283" r:id="rId282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C284" r:id="rId283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C285" r:id="rId284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C286" r:id="rId285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C287" r:id="rId286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C288" r:id="rId287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C289" r:id="rId288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C290" r:id="rId289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C291" r:id="rId290"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C292" r:id="rId291"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C293" r:id="rId292"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C294" r:id="rId293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C295" r:id="rId294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C296" r:id="rId295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C297" r:id="rId296"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C298" r:id="rId297"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C299" r:id="rId298"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C300" r:id="rId299"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C301" r:id="rId300"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C302" r:id="rId301"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C303" r:id="rId302"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C304" r:id="rId303"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C305" r:id="rId304"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C306" r:id="rId305"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C307" r:id="rId306"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C308" r:id="rId307"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C309" r:id="rId308"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C310" r:id="rId309"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C311" r:id="rId310"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C312" r:id="rId311"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C313" r:id="rId312"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C314" r:id="rId313"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C315" r:id="rId314"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C316" r:id="rId315"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C317" r:id="rId316"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C318" r:id="rId317"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C319" r:id="rId318"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C320" r:id="rId319"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C321" r:id="rId320"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C322" r:id="rId321"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C323" r:id="rId322"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C324" r:id="rId323"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C325" r:id="rId324"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C326" r:id="rId325"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C327" r:id="rId326"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C328" r:id="rId327"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C329" r:id="rId328"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C330" r:id="rId329"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C331" r:id="rId330"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C332" r:id="rId331"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C333" r:id="rId332"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C334" r:id="rId333"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C335" r:id="rId334"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C336" r:id="rId335"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C337" r:id="rId336"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C338" r:id="rId337"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C339" r:id="rId338"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C340" r:id="rId339"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C341" r:id="rId340"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C342" r:id="rId341"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C343" r:id="rId342"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C344" r:id="rId343"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C345" r:id="rId344"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C346" r:id="rId345"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C347" r:id="rId346"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C348" r:id="rId347"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C349" r:id="rId348"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C350" r:id="rId349"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C351" r:id="rId350"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C352" r:id="rId351"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C353" r:id="rId352"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C354" r:id="rId353"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C355" r:id="rId354"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C356" r:id="rId355"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C357" r:id="rId356"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C358" r:id="rId357"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C359" r:id="rId358"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C360" r:id="rId359"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C361" r:id="rId360"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C362" r:id="rId361"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C363" r:id="rId362"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C364" r:id="rId363"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C365" r:id="rId364"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C366" r:id="rId365"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C367" r:id="rId366"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C368" r:id="rId367"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C369" r:id="rId368"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C370" r:id="rId369"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C371" r:id="rId370"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C372" r:id="rId371"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C373" r:id="rId372"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C374" r:id="rId373"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C375" r:id="rId374"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C376" r:id="rId375"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C377" r:id="rId376"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C378" r:id="rId377"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C379" r:id="rId378"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C380" r:id="rId379"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C381" r:id="rId380"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C382" r:id="rId381"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C383" r:id="rId382"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C384" r:id="rId383"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C385" r:id="rId384"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C386" r:id="rId385"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C387" r:id="rId386"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C388" r:id="rId387"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C389" r:id="rId388"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Processa lote de 314 links pendentes + fix do HoughLinesP no opencv 5.x
FILA DE TRABALHO/links_pendentes.xlsx: 314 linhas novas marcadas
Processado=X (cod_id, endereco, precisa_confirmar, motivo). 160 delas
ja tinham a coluna Poste preenchida a mao -- usadas como fonte da
verdade direta, sem passar pelo match geometrico (por isso taxa de
baixa confianca caiu bastante nesse lote: ~14% contra ~25% do lote
anterior).

POSTES UTILIZADOS/: 212 em POSTE UTILIZADO - REVISAO, 49 em ESQUINA -
REVISAO, 43 em BAIXA CONFIANCA - REVISAO, 10 arquivos em DUPLICADOS
(colisao de cod_id, aguardando decisao manual).

RELATORIOS/links_postes_processados.xlsx, confirmar_manual.xlsx,
duplicados_para_validar.xlsx: atualizados com o lote acima.

pipeline/run_from_planilha.py: corrige find_pole_x() pra opencv-python
5.x, que mudou o retorno do cv2.HoughLinesP de (N,1,4) pra (N,4) --
sem isso, a deteccao de posicao do poste quebrava com "too many
indices" toda vez que uma linha era encontrada.
</commit_message>
<xml_diff>
--- a/RELATORIOS/confirmar_manual.xlsx
+++ b/RELATORIOS/confirmar_manual.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G389"/>
+  <dimension ref="A1:G435"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -12104,6 +12104,1386 @@
         </is>
       </c>
       <c r="G389" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>223390388</t>
+        </is>
+      </c>
+      <c r="B390" t="n">
+        <v>1444</v>
+      </c>
+      <c r="C390" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5954451,-46.9425453,3a,90y,24.47h,119.42t/data=!3m7!1e1!3m5!1sMAyRGHS2Aeu76z1GhIgysQ!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-29.41673858571123%26panoid%3DMAyRGHS2Aeu76z1GhIgysQ%26yaw%3D24.469471837079002!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D390" t="inlineStr">
+        <is>
+          <t>RUA SACRAMENTO 185, 185, CENTRO</t>
+        </is>
+      </c>
+      <c r="E390" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (6.7m, 51 graus) e rumo (37.5m, 49 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G390" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>220853359</t>
+        </is>
+      </c>
+      <c r="B391" t="n">
+        <v>1447</v>
+      </c>
+      <c r="C391" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5953738,-46.9414941,3a,90y,330.07h,116.91t/data=!3m7!1e1!3m5!1sHqf0_uGbu6JU-x5T30PRhg!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-26.914600177791215%26panoid%3DHqf0_uGbu6JU-x5T30PRhg%26yaw%3D330.0715686499237!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D391" t="inlineStr">
+        <is>
+          <t>PRACA DOUTOR HUGO LEVI 60, 60, CENTRO</t>
+        </is>
+      </c>
+      <c r="E391" t="inlineStr">
+        <is>
+          <t>ATENCAO nome de rua muito diferente: Street View diz o endereco e '184 R. Sacramento', cod_id escolhido e de 'PRACA DOUTOR HUGO LEVI 60, 60, CENTRO' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G391" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>219298347</t>
+        </is>
+      </c>
+      <c r="B392" t="n">
+        <v>1448</v>
+      </c>
+      <c r="C392" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5953361,-46.941184,3a,90y,344.51h,111.4t/data=!3m7!1e1!3m5!1skdmDnao_vIjV75sjTdTJQw!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-21.403687774142966%26panoid%3DkdmDnao_vIjV75sjTdTJQw%26yaw%3D344.5060391339377!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D392" t="inlineStr">
+        <is>
+          <t>PRACA DOUTOR HUGO LEVI 60, 60, CENTRO</t>
+        </is>
+      </c>
+      <c r="E392" t="inlineStr">
+        <is>
+          <t>ATENCAO nome de rua muito diferente: Street View diz o endereco e '218 R. Sacramento', cod_id escolhido e de 'PRACA DOUTOR HUGO LEVI 60, 60, CENTRO' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G392" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>219991693</t>
+        </is>
+      </c>
+      <c r="B393" t="n">
+        <v>1463</v>
+      </c>
+      <c r="C393" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5980166,-46.9418765,3a,35.9y,306.34h,103.47t/data=!3m7!1e1!3m5!1sPi1490SbfEZtjzBU9tqQxQ!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-13.474936902588851%26panoid%3DPi1490SbfEZtjzBU9tqQxQ%26yaw%3D306.3393156827838!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D393" t="inlineStr">
+        <is>
+          <t>AVENIDA PREFEITO ARACELY DE PAULA 1530, 1530, CENTRO</t>
+        </is>
+      </c>
+      <c r="E393" t="inlineStr">
+        <is>
+          <t>confirmar - poste mais proximo (5.0m) tem 170 graus de diferenca de rumo, mas esta perto o suficiente pra ser so ruido de GPS</t>
+        </is>
+      </c>
+      <c r="G393" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>219991677</t>
+        </is>
+      </c>
+      <c r="B394" t="n">
+        <v>1464</v>
+      </c>
+      <c r="C394" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5981139,-46.9418988,3a,41.2y,294.03h,100.6t/data=!3m7!1e1!3m5!1suS_OPDWEM1LTaJ1fxTEpeA!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-10.604436900086114%26panoid%3DuS_OPDWEM1LTaJ1fxTEpeA%26yaw%3D294.02892702923185!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D394" t="inlineStr">
+        <is>
+          <t>RUA SAO CRISTOVAO 10, 10, CENTRO</t>
+        </is>
+      </c>
+      <c r="E394" t="inlineStr">
+        <is>
+          <t>cod_id escolhido pelo rumo, nao pela distancia (mais proximo a 11.0m tinha 104 graus de diferenca de rumo); ATENCAO nome de rua muito diferente: Street View diz o endereco e '349 Av. Pref. Aracely de Paula', cod_id escolhido e de 'RUA SAO CRISTOVAO 10, 10, CENTRO' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G394" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>219991722</t>
+        </is>
+      </c>
+      <c r="B395" t="n">
+        <v>1468</v>
+      </c>
+      <c r="C395" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.598462,-46.942098,3a,48.9y,294.68h,111.46t/data=!3m7!1e1!3m5!1sruZpoLXJzYeIkPvloshhSQ!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-21.458338973602736%26panoid%3DruZpoLXJzYeIkPvloshhSQ%26yaw%3D294.6836964537375!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D395" t="inlineStr">
+        <is>
+          <t>AVENIDA PREFEITO ARACELY DE PAULA 1520, 1520, CENTRO</t>
+        </is>
+      </c>
+      <c r="E395" t="inlineStr">
+        <is>
+          <t>confirmar - poste mais proximo (8.4m) tem 162 graus de diferenca de rumo, mas esta perto o suficiente pra ser so ruido de GPS</t>
+        </is>
+      </c>
+      <c r="G395" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>219298324</t>
+        </is>
+      </c>
+      <c r="B396" t="n">
+        <v>1469</v>
+      </c>
+      <c r="C396" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5986912,-46.9422175,3a,48.9y,304.69h,100.96t/data=!3m7!1e1!3m5!1sB4Q2QS8ocB9CCzxDodSGoA!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-10.964568403133896%26panoid%3DB4Q2QS8ocB9CCzxDodSGoA%26yaw%3D304.68801031693437!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D396" t="inlineStr">
+        <is>
+          <t>AVENIDA PREFEITO ARACELY DE PAULA 1615, 1615, SAO CRISTOVAO</t>
+        </is>
+      </c>
+      <c r="E396" t="inlineStr">
+        <is>
+          <t>confirmar - poste mais proximo (8.5m) tem 175 graus de diferenca de rumo, mas esta perto o suficiente pra ser so ruido de GPS</t>
+        </is>
+      </c>
+      <c r="G396" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>224318357</t>
+        </is>
+      </c>
+      <c r="B397" t="n">
+        <v>1470</v>
+      </c>
+      <c r="C397" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5988588,-46.9422991,3a,32.8y,280.46h,99.48t/data=!3m7!1e1!3m5!1sh0qh8L77nK1vtf3Gmum6pw!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-9.480960739953815%26panoid%3Dh0qh8L77nK1vtf3Gmum6pw%26yaw%3D280.4629864499314!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D397" t="inlineStr">
+        <is>
+          <t>RUA RIO BRANCO 1017, 1017, SAO CRISTOVAO</t>
+        </is>
+      </c>
+      <c r="E397" t="inlineStr">
+        <is>
+          <t>cod_id escolhido pelo rumo, nao pela distancia (mais proximo a 11.2m tinha 120 graus de diferenca de rumo); ATENCAO nome de rua muito diferente: Street View diz o endereco e '1615 Av. Pref. Aracely de Paula', cod_id escolhido e de 'RUA RIO BRANCO 1017, 1017, SAO CRISTOVAO' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G397" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>221621836</t>
+        </is>
+      </c>
+      <c r="B398" t="n">
+        <v>1471</v>
+      </c>
+      <c r="C398" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5993562,-46.9427036,3a,90y,328.45h,115.55t/data=!3m7!1e1!3m5!1sC4KIZsV_448vGdsLknDpMA!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-25.550300710273476%26panoid%3DC4KIZsV_448vGdsLknDpMA%26yaw%3D328.4502335886438!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D398" t="inlineStr">
+        <is>
+          <t>RUA RIO BRANCO 1545, 1545, SAO CRISTOVAO</t>
+        </is>
+      </c>
+      <c r="E398" t="inlineStr">
+        <is>
+          <t>ATENCAO nome de rua muito diferente: Street View diz o endereco e '11 R. Cristóvão Viléla', cod_id escolhido e de 'RUA RIO BRANCO 1545, 1545, SAO CRISTOVAO' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G398" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>219991781</t>
+        </is>
+      </c>
+      <c r="B399" t="n">
+        <v>1472</v>
+      </c>
+      <c r="C399" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5994946,-46.9428295,3a,48.9y,210.43h,111.56t/data=!3m7!1e1!3m5!1sEKm3ziTdWOSxs76LxGAXQA!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-21.557466509447536%26panoid%3DEKm3ziTdWOSxs76LxGAXQA%26yaw%3D210.42652577778694!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D399" t="inlineStr">
+        <is>
+          <t>AVENIDA PREFEITO ARACELY DE PAULA 1535, 1535, SAO CRISTOVAO</t>
+        </is>
+      </c>
+      <c r="E399" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (14.8m, 9 graus) e rumo (36.0m, 5 graus) nao concordam com confianca; ATENCAO nome de rua muito diferente: Street View diz o endereco e '11 R. Cristóvão Viléla', cod_id escolhido e de 'AVENIDA PREFEITO ARACELY DE PAULA 1535, 1535, SAO CRISTOVAO' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G399" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>219298399</t>
+        </is>
+      </c>
+      <c r="B400" t="n">
+        <v>1479</v>
+      </c>
+      <c r="C400" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.6010492,-46.9429766,3a,90y,298.3h,107.66t/data=!3m7!1e1!3m5!1sZoGDMJzbkxxfKaUZxJJN8A!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-17.663268304980022%26panoid%3DZoGDMJzbkxxfKaUZxJJN8A%26yaw%3D298.29835127684316!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D400" t="inlineStr">
+        <is>
+          <t>AVENIDA PREFEITO ARACELY DE PAULA 1385, 1385, JOAO RIBEIRO</t>
+        </is>
+      </c>
+      <c r="E400" t="inlineStr">
+        <is>
+          <t>ATENCAO nome de rua muito diferente: Street View diz o endereco e '470 R. Zéca do Alfredo', cod_id escolhido e de 'AVENIDA PREFEITO ARACELY DE PAULA 1385, 1385, JOAO RIBEIRO' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G400" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>219991799</t>
+        </is>
+      </c>
+      <c r="B401" t="n">
+        <v>1480</v>
+      </c>
+      <c r="C401" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.6012415,-46.9430077,3a,90y,270.38h,126.25t/data=!3m7!1e1!3m5!1s45rVAxIoUIbOLajX_aT21A!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-36.25188369751562%26panoid%3D45rVAxIoUIbOLajX_aT21A%26yaw%3D270.38211733830735!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D401" t="inlineStr">
+        <is>
+          <t>AVENIDA PREFEITO ARACELY DE PAULA 1375, 1375, JOAO RIBEIRO</t>
+        </is>
+      </c>
+      <c r="E401" t="inlineStr">
+        <is>
+          <t>ATENCAO nome de rua muito diferente: Street View diz o endereco e '470 R. Zéca do Alfredo', cod_id escolhido e de 'AVENIDA PREFEITO ARACELY DE PAULA 1375, 1375, JOAO RIBEIRO' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G401" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>223976912</t>
+        </is>
+      </c>
+      <c r="B402" t="n">
+        <v>1494</v>
+      </c>
+      <c r="C402" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5975483,-46.9418027,3a,90y,93.44h,127.52t/data=!3m7!1e1!3m5!1srE5o1vKp63csd-9sdUKwtA!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-37.51571524003353%26panoid%3DrE5o1vKp63csd-9sdUKwtA%26yaw%3D93.43642896738889!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D402" t="inlineStr">
+        <is>
+          <t>RUA HEITOR MONTANDON 113, 113, CENTRO</t>
+        </is>
+      </c>
+      <c r="E402" t="inlineStr">
+        <is>
+          <t>ATENCAO nome de rua muito diferente: Street View diz o endereco e '273 Av. Pref. Aracely de Paula', cod_id escolhido e de 'RUA HEITOR MONTANDON 113, 113, CENTRO' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G402" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>219298400</t>
+        </is>
+      </c>
+      <c r="B403" t="n">
+        <v>1505</v>
+      </c>
+      <c r="C403" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.6001693,-46.9437525,3a,77.2y,213.59h,120.65t/data=!3m7!1e1!3m5!1snc3J8MA-xwEG-t_KIZJohg!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-30.648509274445615%26panoid%3Dnc3J8MA-xwEG-t_KIZJohg%26yaw%3D213.58920650938884!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D403" t="inlineStr">
+        <is>
+          <t>RUA CAMPOS ALTOS 22, 22, SAO CRISTOVAO</t>
+        </is>
+      </c>
+      <c r="E403" t="inlineStr">
+        <is>
+          <t>ATENCAO nome de rua muito diferente: Street View diz o endereco e '99 R. Patrocínio', cod_id escolhido e de 'RUA CAMPOS ALTOS 22, 22, SAO CRISTOVAO' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G403" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>222494683</t>
+        </is>
+      </c>
+      <c r="B404" t="n">
+        <v>1509</v>
+      </c>
+      <c r="C404" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.6008861,-46.9438816,3a,90y,82.69h,119.06t/data=!3m7!1e1!3m5!1ssDLmZqNA30A5ooX1gh0OZA!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-29.060865087836234%26panoid%3DsDLmZqNA30A5ooX1gh0OZA%26yaw%3D82.68857285874853!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D404" t="inlineStr">
+        <is>
+          <t>RUA JOAO MAGALHAES 33, 33, JOAO RIBEIRO</t>
+        </is>
+      </c>
+      <c r="E404" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (0.9m, 65 graus) e rumo (60.4m, 40 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G404" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>224318377</t>
+        </is>
+      </c>
+      <c r="B405" t="n">
+        <v>1513</v>
+      </c>
+      <c r="C405" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.6020409,-46.9438299,3a,48.9y,24.97h,111.95t/data=!3m7!1e1!3m5!1sPzUGIhHS54oqfQviguauTA!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-21.948685384903797%26panoid%3DPzUGIhHS54oqfQviguauTA%26yaw%3D24.970279946775108!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D405" t="inlineStr">
+        <is>
+          <t>RUA JOAO MAGALHAES 164, 164, JOAO RIBEIRO</t>
+        </is>
+      </c>
+      <c r="E405" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (15.9m, 34 graus) e rumo (44.9m, 21 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G405" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>224318385</t>
+        </is>
+      </c>
+      <c r="B406" t="n">
+        <v>1514</v>
+      </c>
+      <c r="C406" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.6022323,-46.9438292,3a,90y,97.22h,120.81t/data=!3m7!1e1!3m5!1s5hprhny6ZNmKGo3CoXQmWg!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-30.808186557884156%26panoid%3D5hprhny6ZNmKGo3CoXQmWg%26yaw%3D97.2240229118285!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D406" t="inlineStr">
+        <is>
+          <t>RUA JOAO MAGALHAES 178, 178, JOAO RIBEIRO</t>
+        </is>
+      </c>
+      <c r="E406" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (3.4m, 131 graus) e rumo (49.4m, 72 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G406" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>223455631</t>
+        </is>
+      </c>
+      <c r="B407" t="n">
+        <v>1533</v>
+      </c>
+      <c r="C407" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.59536,-46.9397019,3a,75y,347.54h,113.83t/data=!3m7!1e1!3m5!1s5RVb8a1tmuGZj6BElnERQA!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-23.834929177587256%26panoid%3D5RVb8a1tmuGZj6BElnERQA%26yaw%3D347.5371082612378!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D407" t="inlineStr">
+        <is>
+          <t>RUA DOM BOSCO 153, 153, CENTRO</t>
+        </is>
+      </c>
+      <c r="E407" t="inlineStr">
+        <is>
+          <t>confirmar - poste mais proximo (8.6m) tem 130 graus de diferenca de rumo, mas esta perto o suficiente pra ser so ruido de GPS</t>
+        </is>
+      </c>
+      <c r="G407" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>224357790</t>
+        </is>
+      </c>
+      <c r="B408" t="n">
+        <v>1556</v>
+      </c>
+      <c r="C408" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5969409,-46.9377501,3a,57.4y,332.37h,107.09t/data=!3m7!1e1!3m5!1sXBOiiRBTq2UVZw6JXN_vpA!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-17.08856862324427%26panoid%3DXBOiiRBTq2UVZw6JXN_vpA%26yaw%3D332.36617584947896!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D408" t="inlineStr">
+        <is>
+          <t>RUA MARIA RITA DE AGUIAR 18, 18, CENTRO</t>
+        </is>
+      </c>
+      <c r="E408" t="inlineStr">
+        <is>
+          <t>ATENCAO nome de rua muito diferente: Street View diz o endereco e '325 R. Francelino Cardoso', cod_id escolhido e de 'RUA MARIA RITA DE AGUIAR 18, 18, CENTRO' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G408" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>2683729726</t>
+        </is>
+      </c>
+      <c r="B409" t="n">
+        <v>1559</v>
+      </c>
+      <c r="C409" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5970289,-46.9376445,3a,90y,36.42h,122.59t/data=!3m7!1e1!3m5!1sDP13BIPmUSQL4QfkuQskgA!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-32.58835488021839%26panoid%3DDP13BIPmUSQL4QfkuQskgA%26yaw%3D36.417788848836!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D409" t="inlineStr">
+        <is>
+          <t>RUA FRANCELINO CARDOSO 325, 325, CENTRO</t>
+        </is>
+      </c>
+      <c r="E409" t="inlineStr">
+        <is>
+          <t>ATENCAO nome de rua muito diferente: Street View diz o endereco e '2 R. Maria Rita de Águiar', cod_id escolhido e de 'RUA FRANCELINO CARDOSO 325, 325, CENTRO' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G409" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>224357795</t>
+        </is>
+      </c>
+      <c r="B410" t="n">
+        <v>1564</v>
+      </c>
+      <c r="C410" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5971055,-46.938578,3a,90y,21.17h,112.97t/data=!3m7!1e1!3m5!1sUsz1Rhtge8LcK1IYkewOvA!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-22.970616935349%26panoid%3DUsz1Rhtge8LcK1IYkewOvA%26yaw%3D21.1693190619092!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D410" t="inlineStr">
+        <is>
+          <t>RUA PRIMEIRO DE MAIO 177, 177, CENTRO</t>
+        </is>
+      </c>
+      <c r="E410" t="inlineStr">
+        <is>
+          <t>confirmar - poste mais proximo (5.3m) tem 76 graus de diferenca de rumo, mas esta perto o suficiente pra ser so ruido de GPS; ATENCAO nome de rua muito diferente: Street View diz o endereco e '334 R. Maria Rita de Águiar', cod_id escolhido e de 'RUA PRIMEIRO DE MAIO 177, 177, CENTRO' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G410" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>220854122</t>
+        </is>
+      </c>
+      <c r="B411" t="n">
+        <v>1565</v>
+      </c>
+      <c r="C411" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.59713,-46.9388865,3a,90y,353.05h,123.51t/data=!3m7!1e1!3m5!1sv6w1s3iufMsQCZ_f7RUjJg!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-33.50736237778975%26panoid%3Dv6w1s3iufMsQCZ_f7RUjJg%26yaw%3D353.04822879284575!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D411" t="inlineStr">
+        <is>
+          <t>RUA PRIMEIRO DE MAIO 177, 177, CENTRO</t>
+        </is>
+      </c>
+      <c r="E411" t="inlineStr">
+        <is>
+          <t>ATENCAO nome de rua muito diferente: Street View diz o endereco e '334 R. Maria Rita de Águiar', cod_id escolhido e de 'RUA PRIMEIRO DE MAIO 177, 177, CENTRO' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G411" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>219992975</t>
+        </is>
+      </c>
+      <c r="B412" t="n">
+        <v>1569</v>
+      </c>
+      <c r="C412" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5972595,-46.9403027,3a,75y,297.29h,112.28t/data=!3m7!1e1!3m5!1s98oBFA94N7oRg7M-mpWGnw!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-22.27961692712408%26panoid%3D98oBFA94N7oRg7M-mpWGnw%26yaw%3D297.28841972816076!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D412" t="inlineStr">
+        <is>
+          <t>AVENIDA IMBIARA 387, 387, CENTRO</t>
+        </is>
+      </c>
+      <c r="E412" t="inlineStr">
+        <is>
+          <t>ATENCAO nome de rua muito diferente: Street View diz o endereco e '234 R. Maria Rita de Águiar', cod_id escolhido e de 'AVENIDA IMBIARA 387, 387, CENTRO' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G412" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>222494582</t>
+        </is>
+      </c>
+      <c r="B413" t="n">
+        <v>1586</v>
+      </c>
+      <c r="C413" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5962966,-46.9407178,3a,63.6y,330.63h,114.43t/data=!3m7!1e1!3m5!1sjDOyHhewvLTAvNQIGxg5Rg!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-24.433278959289254%26panoid%3DjDOyHhewvLTAvNQIGxg5Rg%26yaw%3D330.62778566786966!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D413" t="inlineStr">
+        <is>
+          <t>AVENIDA IMBIARA 260, 260, CENTRO</t>
+        </is>
+      </c>
+      <c r="E413" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (10.6m, 18 graus) e rumo (46.5m, 17 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G413" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>224318231</t>
+        </is>
+      </c>
+      <c r="B414" t="n">
+        <v>1590</v>
+      </c>
+      <c r="C414" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5974873,-46.9405985,3a,48.9y,207.49h,121.64t/data=!3m7!1e1!3m5!1s4QWWyzTpHNdNFndcD7M4Xg!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-31.64332512248778%26panoid%3D4QWWyzTpHNdNFndcD7M4Xg%26yaw%3D207.48679758334757!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D414" t="inlineStr">
+        <is>
+          <t>AVENIDA IMBIARA 444, 444, CENTRO</t>
+        </is>
+      </c>
+      <c r="E414" t="inlineStr">
+        <is>
+          <t>ATENCAO nome de rua muito diferente: Street View diz o endereco e '432 BR-452', cod_id escolhido e de 'AVENIDA IMBIARA 444, 444, CENTRO' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G414" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>219298258</t>
+        </is>
+      </c>
+      <c r="B415" t="n">
+        <v>1591</v>
+      </c>
+      <c r="C415" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5978472,-46.940567,3a,48.9y,200.74h,121.12t/data=!3m7!1e1!3m5!1sbj0IUPLQg1F9mdRfOe_gkw!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-31.116267524035777%26panoid%3Dbj0IUPLQg1F9mdRfOe_gkw%26yaw%3D200.74161848859035!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D415" t="inlineStr">
+        <is>
+          <t>AVENIDA IMBIARA 494, 494, CENTRO</t>
+        </is>
+      </c>
+      <c r="E415" t="inlineStr">
+        <is>
+          <t>ATENCAO nome de rua muito diferente: Street View diz o endereco e '482 BR-452', cod_id escolhido e de 'AVENIDA IMBIARA 494, 494, CENTRO' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G415" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>220780206</t>
+        </is>
+      </c>
+      <c r="B416" t="n">
+        <v>1596</v>
+      </c>
+      <c r="C416" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.5997242,-46.9403877,3a,90y,214.69h,132.87t/data=!3m7!1e1!3m5!1sEelXBcFc4YImbepO3m7eig!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-42.86679626398242%26panoid%3DEelXBcFc4YImbepO3m7eig%26yaw%3D214.69121569513172!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D416" t="inlineStr">
+        <is>
+          <t>AVENIDA IMBIARA 665, 665, CENTRO</t>
+        </is>
+      </c>
+      <c r="E416" t="inlineStr">
+        <is>
+          <t>ATENCAO nome de rua muito diferente: Street View diz o endereco e '620 MG-428', cod_id escolhido e de 'AVENIDA IMBIARA 665, 665, CENTRO' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G416" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>224318209</t>
+        </is>
+      </c>
+      <c r="B417" t="n">
+        <v>1597</v>
+      </c>
+      <c r="C417" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.6000416,-46.9403588,3a,90y,249.87h,134.99t/data=!3m7!1e1!3m5!1sOanHs3-t6SRzU-2cmn6Apw!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-44.987133821041%26panoid%3DOanHs3-t6SRzU-2cmn6Apw%26yaw%3D249.87270478397892!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D417" t="inlineStr">
+        <is>
+          <t>AVENIDA IMBIARA 754, 754, JOAO RIBEIRO</t>
+        </is>
+      </c>
+      <c r="E417" t="inlineStr">
+        <is>
+          <t>ATENCAO nome de rua muito diferente: Street View diz o endereco e '779 MG-428', cod_id escolhido e de 'AVENIDA IMBIARA 754, 754, JOAO RIBEIRO' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G417" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>221621722</t>
+        </is>
+      </c>
+      <c r="B418" t="n">
+        <v>1602</v>
+      </c>
+      <c r="C418" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.6017136,-46.9402054,3a,90y,209.4h,131.85t/data=!3m7!1e1!3m5!1s3iSYsrhFfINUn2taY1HUEQ!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-41.85453531185149%26panoid%3D3iSYsrhFfINUn2taY1HUEQ%26yaw%3D209.40387396709974!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D418" t="inlineStr">
+        <is>
+          <t>AVENIDA IMBIARA 990, 990, JOAO RIBEIRO</t>
+        </is>
+      </c>
+      <c r="E418" t="inlineStr">
+        <is>
+          <t>ATENCAO nome de rua muito diferente: Street View diz o endereco e '990 BR-452', cod_id escolhido e de 'AVENIDA IMBIARA 990, 990, JOAO RIBEIRO' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G418" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>222494577</t>
+        </is>
+      </c>
+      <c r="B419" t="n">
+        <v>1609</v>
+      </c>
+      <c r="C419" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.6037802,-46.9401254,3a,90y,315.19h,138.09t/data=!3m7!1e1!3m5!1scUmOCK205ceEuTsFMz5k2w!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-48.087911328270536%26panoid%3DcUmOCK205ceEuTsFMz5k2w%26yaw%3D315.1938239894892!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D419" t="inlineStr">
+        <is>
+          <t>AVENIDA IMBIARA 1212, 1212, JOAO RIBEIRO</t>
+        </is>
+      </c>
+      <c r="E419" t="inlineStr">
+        <is>
+          <t>ATENCAO nome de rua muito diferente: Street View diz o endereco e '1170 MG-428', cod_id escolhido e de 'AVENIDA IMBIARA 1212, 1212, JOAO RIBEIRO' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G419" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>219991635</t>
+        </is>
+      </c>
+      <c r="B420" t="n">
+        <v>1610</v>
+      </c>
+      <c r="C420" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.6039617,-46.9401272,3a,90y,267.42h,140.53t/data=!3m7!1e1!3m5!1syhNmmEa6uQhX_rjw4p2BTA!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-50.52661235290648%26panoid%3DyhNmmEa6uQhX_rjw4p2BTA%26yaw%3D267.42224532145354!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D420" t="inlineStr">
+        <is>
+          <t>RUA CELIDONIO AFONSECA E SILVA 56, 56, JOAO RIBEIRO</t>
+        </is>
+      </c>
+      <c r="E420" t="inlineStr">
+        <is>
+          <t>ATENCAO nome de rua muito diferente: Street View diz o endereco e '1212 MG-428', cod_id escolhido e de 'RUA CELIDONIO AFONSECA E SILVA 56, 56, JOAO RIBEIRO' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G420" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>219298241</t>
+        </is>
+      </c>
+      <c r="B421" t="n">
+        <v>1617</v>
+      </c>
+      <c r="C421" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.60538,-46.940116,3a,90y,257.21h,136.23t/data=!3m7!1e1!3m5!1sPQYs4xaAXfUehEjXPrCFwg!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-46.22807801633718%26panoid%3DPQYs4xaAXfUehEjXPrCFwg%26yaw%3D257.21477128253895!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D421" t="inlineStr">
+        <is>
+          <t>AVENIDA IMBIARA 1423, 1423, SILVERIA</t>
+        </is>
+      </c>
+      <c r="E421" t="inlineStr">
+        <is>
+          <t>ATENCAO nome de rua muito diferente: Street View diz o endereco e '1400 BR-146', cod_id escolhido e de 'AVENIDA IMBIARA 1423, 1423, SILVERIA' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G421" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>223977809</t>
+        </is>
+      </c>
+      <c r="B422" t="n">
+        <v>1625</v>
+      </c>
+      <c r="C422" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.6003177,-46.9396134,3a,75y,294.49h,115.92t/data=!3m7!1e1!3m5!1s8ZPLP0MBi2wBf96gyKG7aA!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-25.918330390989894%26panoid%3D8ZPLP0MBi2wBf96gyKG7aA%26yaw%3D294.48660561770976!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D422" t="inlineStr">
+        <is>
+          <t>RUA URBANO VILELA 62, 62, CENTRO</t>
+        </is>
+      </c>
+      <c r="E422" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (12.8m, 20 graus) e rumo (58.1m, 17 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G422" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>219090471</t>
+        </is>
+      </c>
+      <c r="B423" t="n">
+        <v>1630</v>
+      </c>
+      <c r="C423" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.6007244,-46.9415228,3a,90y,51.51h,122.43t/data=!3m7!1e1!3m5!1smy04BL8GpMSlutBBwPIPbQ!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-32.43005273570127%26panoid%3Dmy04BL8GpMSlutBBwPIPbQ%26yaw%3D51.50751890793638!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D423" t="inlineStr">
+        <is>
+          <t>RUA BENEDITO SIMOES BORGES 30, 30, JOAO RIBEIRO</t>
+        </is>
+      </c>
+      <c r="E423" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (4.1m, 51 graus) e rumo (42.3m, 50 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G423" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>220780278</t>
+        </is>
+      </c>
+      <c r="B424" t="n">
+        <v>1632</v>
+      </c>
+      <c r="C424" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.6013958,-46.9414574,3a,90y,115.43h,112.92t/data=!3m7!1e1!3m5!1s84qroBi2VYqvU4JKZ1rzng!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-22.915309653647356%26panoid%3D84qroBi2VYqvU4JKZ1rzng%26yaw%3D115.43423627644611!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D424" t="inlineStr">
+        <is>
+          <t>RUA JOAO BATISTA FERNANDES 110, 110, JOAO RIBEIRO</t>
+        </is>
+      </c>
+      <c r="E424" t="inlineStr">
+        <is>
+          <t>ATENCAO nome de rua muito diferente: Street View diz o endereco e '60 R. Benedito Simões Borges', cod_id escolhido e de 'RUA JOAO BATISTA FERNANDES 110, 110, JOAO RIBEIRO' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G424" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>221621764</t>
+        </is>
+      </c>
+      <c r="B425" t="n">
+        <v>1636</v>
+      </c>
+      <c r="C425" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.6010184,-46.9420432,3a,90y,68.1h,135.49t/data=!3m7!1e1!3m5!1sFjk7xjg8oC3NE1vF1ywnEw!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-45.493613478948646%26panoid%3DFjk7xjg8oC3NE1vF1ywnEw%26yaw%3D68.10278578146611!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D425" t="inlineStr">
+        <is>
+          <t>RUA JOAO RIBEIRO 84, 84, JOAO RIBEIRO</t>
+        </is>
+      </c>
+      <c r="E425" t="inlineStr">
+        <is>
+          <t>confirmar - poste mais proximo (1.0m) tem 161 graus de diferenca de rumo, mas esta perto o suficiente pra ser so ruido de GPS</t>
+        </is>
+      </c>
+      <c r="G425" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>223976935</t>
+        </is>
+      </c>
+      <c r="B426" t="n">
+        <v>1638</v>
+      </c>
+      <c r="C426" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.6003507,-46.9421086,3a,75y,121.12h,120.57t/data=!3m7!1e1!3m5!1sUHPcCirwSyOstR381pJAVw!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-30.56815856888572%26panoid%3DUHPcCirwSyOstR381pJAVw%26yaw%3D121.11636216480419!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D426" t="inlineStr">
+        <is>
+          <t>RUA PAUL HARRIS 197, 197, JOAO RIBEIRO</t>
+        </is>
+      </c>
+      <c r="E426" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (5.5m, 60 graus) e rumo (48.9m, 31 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G426" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>223976927</t>
+        </is>
+      </c>
+      <c r="B427" t="n">
+        <v>1644</v>
+      </c>
+      <c r="C427" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.6020604,-46.941106,3a,90y,214.6h,131.63t/data=!3m7!1e1!3m5!1sFXE3XvlhIs1Gw41do2ZPBA!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-41.62961189030733%26panoid%3DFXE3XvlhIs1Gw41do2ZPBA%26yaw%3D214.60131405544652!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D427" t="inlineStr">
+        <is>
+          <t>RUA ACHILES NOLLI 80, 80, JOAO RIBEIRO</t>
+        </is>
+      </c>
+      <c r="E427" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (6.9m, 35 graus) e rumo (45.7m, 31 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G427" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>219298289</t>
+        </is>
+      </c>
+      <c r="B428" t="n">
+        <v>1646</v>
+      </c>
+      <c r="C428" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.6024131,-46.9408195,3a,90y,140.06h,127.38t/data=!3m7!1e1!3m5!1sHpQkeel_-aRsS3HBAkn5LA!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-37.381276050104745%26panoid%3DHpQkeel_-aRsS3HBAkn5LA%26yaw%3D140.06220466606095!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D428" t="inlineStr">
+        <is>
+          <t>RUA CLAUDIO JOSE DE FARIA 0, 0, JOAO RIBEIRO</t>
+        </is>
+      </c>
+      <c r="E428" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (4.7m, 78 graus) e rumo (63.0m, 49 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G428" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>219386943</t>
+        </is>
+      </c>
+      <c r="B429" t="n">
+        <v>1650</v>
+      </c>
+      <c r="C429" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.6034622,-46.9409972,3a,90y,252.42h,141.35t/data=!3m7!1e1!3m5!1s_CEyjT-cyaZWi7tKxx6mIw!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-51.345627462858204%26panoid%3D_CEyjT-cyaZWi7tKxx6mIw%26yaw%3D252.42313123536246!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D429" t="inlineStr">
+        <is>
+          <t>RUA WANTUIR BATISTA DA COSTA 115, 115, JOAO RIBEIRO</t>
+        </is>
+      </c>
+      <c r="E429" t="inlineStr">
+        <is>
+          <t>ATENCAO nome de rua muito diferente: Street View diz o endereco e '300 R. Achiles Noli', cod_id escolhido e de 'RUA WANTUIR BATISTA DA COSTA 115, 115, JOAO RIBEIRO' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G429" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>221621776</t>
+        </is>
+      </c>
+      <c r="B430" t="n">
+        <v>1661</v>
+      </c>
+      <c r="C430" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.6023358,-46.9420981,3a,66.8y,33.46h,127.89t/data=!3m7!1e1!3m5!1strPZYt-lXoQ_WPmGpOqTUA!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-37.88771603236425%26panoid%3DtrPZYt-lXoQ_WPmGpOqTUA%26yaw%3D33.46096636880882!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D430" t="inlineStr">
+        <is>
+          <t>RUA JOAO RIBEIRO 204, 204, JOAO RIBEIRO</t>
+        </is>
+      </c>
+      <c r="E430" t="inlineStr">
+        <is>
+          <t>ATENCAO nome de rua muito diferente: Street View diz o endereco e '1263 Av. Pref. Aracely de Paula', cod_id escolhido e de 'RUA JOAO RIBEIRO 204, 204, JOAO RIBEIRO' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G430" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>222494684</t>
+        </is>
+      </c>
+      <c r="B431" t="n">
+        <v>1669</v>
+      </c>
+      <c r="C431" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.6018009,-46.9429931,3a,33.5y,188.57h,95.13t/data=!3m7!1e1!3m5!1sDhB_MB5-h2Ut2Zky-Z66Nw!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-5.132276596765649%26panoid%3DDhB_MB5-h2Ut2Zky-Z66Nw%26yaw%3D188.56766440933848!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D431" t="inlineStr">
+        <is>
+          <t>RUA ZECA DO ALFREDO 0, 0, JOAO RIBEIRO</t>
+        </is>
+      </c>
+      <c r="E431" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (10.8m, 14 graus) e rumo (50.2m, 6 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G431" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>221621792</t>
+        </is>
+      </c>
+      <c r="B432" t="n">
+        <v>1688</v>
+      </c>
+      <c r="C432" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.604117,-46.9429183,3a,90y,199.66h,117.39t/data=!3m7!1e1!3m5!1sWdl3eZkglo46BiZupGzdCA!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-27.39471923369092%26panoid%3DWdl3eZkglo46BiZupGzdCA%26yaw%3D199.66086884371234!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D432" t="inlineStr">
+        <is>
+          <t>RUA ZECA DO ALFREDO 348, 348, JOAO RIBEIRO</t>
+        </is>
+      </c>
+      <c r="E432" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (10.8m, 8 graus) e rumo (36.1m, 3 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G432" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>223976966</t>
+        </is>
+      </c>
+      <c r="B433" t="n">
+        <v>1701</v>
+      </c>
+      <c r="C433" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.6050138,-46.9417413,3a,63.6y,197.26h,110.48t/data=!3m7!1e1!3m5!1sgHK7JUerHfCCYEuzyXTxjw!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-20.481942692708785%26panoid%3DgHK7JUerHfCCYEuzyXTxjw%26yaw%3D197.25664495821502!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D433" t="inlineStr">
+        <is>
+          <t>RUA DONATO PINHEIRO DOS SANTOS 166, 166, JOAO RIBEIRO</t>
+        </is>
+      </c>
+      <c r="E433" t="inlineStr">
+        <is>
+          <t>ATENCAO nome de rua muito diferente: Street View diz o endereco e '477 R. João Ribeiro', cod_id escolhido e de 'RUA DONATO PINHEIRO DOS SANTOS 166, 166, JOAO RIBEIRO' - conferir manualmente (nao troquei sozinho, pode ser esquina ou so grafia diferente)</t>
+        </is>
+      </c>
+      <c r="G433" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>222494703</t>
+        </is>
+      </c>
+      <c r="B434" t="n">
+        <v>1709</v>
+      </c>
+      <c r="C434" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.6063065,-46.943692,3a,90y,116.35h,136.63t/data=!3m7!1e1!3m5!1s7NMuY9v2-rnRxNfblNndeg!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-46.62514707671832%26panoid%3D7NMuY9v2-rnRxNfblNndeg%26yaw%3D116.34823733733165!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D434" t="inlineStr">
+        <is>
+          <t>RUA JOSE BARBOSA DE CASTRO 62, 62, FERTIZA</t>
+        </is>
+      </c>
+      <c r="E434" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (3.6m, 39 graus) e rumo (34.8m, 32 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G434" t="inlineStr">
+        <is>
+          <t>BAIXA CONFIANCA - REVISAO</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>219298365</t>
+        </is>
+      </c>
+      <c r="B435" t="n">
+        <v>1712</v>
+      </c>
+      <c r="C435" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/@-19.6074252,-46.943442,3a,75y,22.83h,116.06t/data=!3m7!1e1!3m5!1sgb2mi-tX9jk-6EXR_AKWYw!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-26.055745226802742%26panoid%3Dgb2mi-tX9jk-6EXR_AKWYw%26yaw%3D22.82847751255779!7i16384!8i8192?entry=ttu&amp;g_ep=EgoyMDI2MDgxOS4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="D435" t="inlineStr">
+        <is>
+          <t>RUA JOSE BARBOSA DE CASTRO 156, 156, FERTIZA</t>
+        </is>
+      </c>
+      <c r="E435" t="inlineStr">
+        <is>
+          <t>confirmar - distancia (7.9m, 45 graus) e rumo (87.2m, 36 graus) nao concordam com confianca</t>
+        </is>
+      </c>
+      <c r="G435" t="inlineStr">
         <is>
           <t>BAIXA CONFIANCA - REVISAO</t>
         </is>
@@ -12499,6 +13879,52 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C387" r:id="rId386"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C388" r:id="rId387"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C389" r:id="rId388"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C390" r:id="rId389"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C391" r:id="rId390"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C392" r:id="rId391"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C393" r:id="rId392"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C394" r:id="rId393"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C395" r:id="rId394"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C396" r:id="rId395"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C397" r:id="rId396"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C398" r:id="rId397"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C399" r:id="rId398"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C400" r:id="rId399"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C401" r:id="rId400"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C402" r:id="rId401"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C403" r:id="rId402"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C404" r:id="rId403"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C405" r:id="rId404"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C406" r:id="rId405"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C407" r:id="rId406"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C408" r:id="rId407"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C409" r:id="rId408"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C410" r:id="rId409"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C411" r:id="rId410"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C412" r:id="rId411"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C413" r:id="rId412"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C414" r:id="rId413"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C415" r:id="rId414"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C416" r:id="rId415"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C417" r:id="rId416"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C418" r:id="rId417"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C419" r:id="rId418"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C420" r:id="rId419"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C421" r:id="rId420"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C422" r:id="rId421"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C423" r:id="rId422"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C424" r:id="rId423"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C425" r:id="rId424"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C426" r:id="rId425"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C427" r:id="rId426"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C428" r:id="rId427"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C429" r:id="rId428"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C430" r:id="rId429"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C431" r:id="rId430"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C432" r:id="rId431"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C433" r:id="rId432"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C434" r:id="rId433"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C435" r:id="rId434"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>